<commit_message>
Adiciona aluna Jaqueline Galo (treinos A, B, C)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -736,6 +736,53 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Plano de treino · 3x por semana</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Iniciante · Treinos A, B e C</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>GANHO DE MASSA MUSCULAR</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Iniciante com foco em ganho de massa muscular, treinando 3x por semana. Treinos A (inferiores), B (costas, ombro e glúteos) e C (abdômen, tríceps e pernas). Técnica antes da carga e progressão gradual semana a semana. Início em 01/06/2025.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -747,7 +794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2274,13 +2321,11 @@
           <t>800 m</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>Intervalado: correr forte cada tiro de 800 m e recuperar entre eles. Foco no controle respiratório.</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2318,9 +2363,6 @@
           <t>15</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2358,13 +2400,11 @@
           <t>12</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>Elástico nas pernas, joelhos altos e cadência rápida.</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2402,13 +2442,11 @@
           <t>20</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
           <t>Pés afastados e pontas para fora; descer com os joelhos alinhados.</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2446,13 +2484,771 @@
           <t>15</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>Aterrissar suave, amortecendo com os joelhos.</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>A · Inferiores</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Aquecimento · 10 min de escada</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Aquecimento</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>10 min</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>A · Inferiores</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Agachamento sumô com halteres</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Pernas/glúteos</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Progressão de carga: 5 → 7 → 10 → 12 kg ao longo das séries.</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>A · Inferiores</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Leg press</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Pernas</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>15/12/10</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Drop set: reduzir a carga a cada parada.</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>A · Inferiores</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Stiff com halteres</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Posterior/glúteo</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Descida lenta (controlada). Carga: 2 halteres de 5 kg.</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>A · Inferiores</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Cadeira extensora</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Quadríceps</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>20/20/15/15</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Progressão de carga ao longo das séries.</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>A · Inferiores</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Avanço livre no step</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Pernas/glúteos</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Sem carga (peso do corpo).</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>B · Costas, Ombro e Glúteos</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Puxador frente (pegada delta)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Dorsais · principal</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>20/15/12/10</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Progressão de carga ao longo das séries. Pegada delta (triângulo).</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>B · Costas, Ombro e Glúteos</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Remada unilateral na polia alta</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>B · Costas, Ombro e Glúteos</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Cadeira abdutora</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Glúteos · abdutores</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>20/15/12/10</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Progressão de carga ao longo das séries.</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>B · Costas, Ombro e Glúteos</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Elevação pélvica no step</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Glúteos</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>B · Costas, Ombro e Glúteos</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Glúteo chute no pulley</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Glúteos</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>C · Abdômen, Tríceps e Pernas</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Remada na polia média</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>C · Abdômen, Tríceps e Pernas</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Tríceps pulley</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Tríceps</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>C · Abdômen, Tríceps e Pernas</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Desenvolvimento</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Ombro</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Carga: 4 kg.</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>C · Abdômen, Tríceps e Pernas</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Agachamento sumô</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Pernas/glúteos</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>15/15/12/12</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Progressão de carga ao longo das séries.</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>C · Abdômen, Tríceps e Pernas</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Leg press</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Pernas</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>C · Abdômen, Tríceps e Pernas</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Abdominal curto</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Contraia o abdômen no topo.</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>C · Abdômen, Tríceps e Pernas</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Prancha isométrica</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>30s</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Corpo alinhado, core contraído.</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Completa perfil da Jaqueline com dados da avaliacao fisica
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -749,7 +749,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Iniciante · Treinos A, B e C</t>
+          <t>Iniciante · Treinos A, B e C · Início 01/06/2025</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -759,12 +759,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Iniciante com foco em ganho de massa muscular, treinando 3x por semana. Treinos A (inferiores), B (costas, ombro e glúteos) e C (abdômen, tríceps e pernas). Técnica antes da carga e progressão gradual semana a semana. Início em 01/06/2025.</t>
+          <t>Iniciante, treinando 3x por semana com foco em ganho de massa muscular. Evolução excelente desde 20/05/2025: de 78,1 kg e 32,7% de gordura para 64,2 kg e 18,8% (07/05/2026) — cerca de 14 kg de gordura a menos mantendo a massa magra (~52 kg) e 9,5 cm de cintura reduzidos. Meta: 60 kg e 18% de gordura. Agora o foco é ganhar massa muscular com técnica impecável e progressão gradual.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>Junho/2026</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2516,15 +2516,11 @@
           <t>Aquecimento</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
           <t>10 min</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2562,13 +2558,11 @@
           <t>15</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
           <t>Progressão de carga: 5 → 7 → 10 → 12 kg ao longo das séries.</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2606,13 +2600,11 @@
           <t>15/12/10</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>Drop set: reduzir a carga a cada parada.</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2650,13 +2642,11 @@
           <t>12</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>Descida lenta (controlada). Carga: 2 halteres de 5 kg.</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2694,13 +2684,11 @@
           <t>20/20/15/15</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>Progressão de carga ao longo das séries.</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2738,13 +2726,11 @@
           <t>15</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
           <t>Sem carga (peso do corpo).</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2782,13 +2768,11 @@
           <t>20/15/12/10</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
           <t>Progressão de carga ao longo das séries. Pegada delta (triângulo).</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2826,9 +2810,6 @@
           <t>15</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2866,13 +2847,11 @@
           <t>20/15/12/10</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>Progressão de carga ao longo das séries.</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2910,9 +2889,6 @@
           <t>15</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2950,9 +2926,6 @@
           <t>12</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2990,9 +2963,6 @@
           <t>15</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3030,9 +3000,6 @@
           <t>15</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3070,13 +3037,11 @@
           <t>12</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
           <t>Carga: 4 kg.</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3114,13 +3079,11 @@
           <t>15/15/12/12</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>Progressão de carga ao longo das séries.</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3158,9 +3121,6 @@
           <t>15</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3198,13 +3158,11 @@
           <t>20</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>Contraia o abdômen no topo.</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3242,13 +3200,11 @@
           <t>30s</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
           <t>Corpo alinhado, core contraído.</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Atualiza Jaqueline: objetivo (hipertrofia) e metas do trimestre
Gerador agora aceita coluna metas na aba Alunos (metas por aluno).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -594,6 +594,11 @@
           <t>prs</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>metas</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -749,7 +754,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Iniciante · Treinos A, B e C · Início 01/06/2025</t>
+          <t>Foco: ganho de massa muscular · Treinos A, B e C</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -759,7 +764,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Iniciante, treinando 3x por semana com foco em ganho de massa muscular. Evolução excelente desde 20/05/2025: de 78,1 kg e 32,7% de gordura para 64,2 kg e 18,8% (07/05/2026) — cerca de 14 kg de gordura a menos mantendo a massa magra (~52 kg) e 9,5 cm de cintura reduzidos. Meta: 60 kg e 18% de gordura. Agora o foco é ganhar massa muscular com técnica impecável e progressão gradual.</t>
+          <t>Evolução excelente desde 05/2025: saiu de 32% para 18,8% de gordura, com ótima recomposição corporal. Não está mais na fase inicial — agora o foco é o ganho de massa muscular, com técnica impecável e progressão de carga. Treinos A (inferiores), B (costas, ombro e glúteos) e C (abdômen, tríceps e pernas).</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -774,12 +779,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0/8</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Não medido</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Ganhar 500 g de massa muscular=0; Agachamento sumô com 20 kg=0; Fazer 8 treinos no mês=0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Troca 1RM estimado por avaliacao fisica (composicao + circunferencias)
- Remove cards/numeros de 1RM estimado do topo, painel inicial e Evolucao
- Nova aba Avaliacao na planilha: composicao corporal e circunferencias,
  com inicio -> atual + meta, por aluna
- Gerador injeta os dados reais; alunas sem avaliacao mantem o layout exemplo
- Preenche a avaliacao da Jaqueline (evolucao desde 05/2025)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Alunos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Treinos" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Biblioteca" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Avaliacao" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3305,4 +3306,372 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>aluno</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>secao</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>metrica</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>unidade</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>inicio</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>atual</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>direcao</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Composição</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Peso</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>78,1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>64,2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Composição</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>% Gordura</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>32,66</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>18,77</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Composição</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Massa magra</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>52,58</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>52,15</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Composição</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Gordura (kg)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>25,51</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>12,05</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Circunferências</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Cintura</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>75,5</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Circunferências</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Abdômen</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>99,5</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Circunferências</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Braço</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>33,5</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>29,5</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Circunferências</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Coxa</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>61,5</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>alto</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ajustes de cabecalho e planos
Remove a foto da treinadora (HTML+CSS); logo maior (72->110px); nome do cliente centralizado; planos padronizados em 3 meses e 6 meses.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -609,7 +609,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Plano Premium · 12ª semana</t>
+          <t>Plano 6 meses</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Plano Essencial · 4ª semana</t>
+          <t>Plano 3 meses</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Plano de treino · em andamento</t>
+          <t>Plano 6 meses</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Plano de treino · 3x por semana</t>
+          <t>Plano 3 meses</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3474,7 +3474,6 @@
           <t>52,15</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>alto</t>
@@ -3512,7 +3511,6 @@
           <t>12,05</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>baixo</t>
@@ -3550,7 +3548,6 @@
           <t>75,5</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>baixo</t>
@@ -3588,7 +3585,6 @@
           <t>84</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>baixo</t>
@@ -3626,7 +3622,6 @@
           <t>29,5</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>alto</t>
@@ -3664,7 +3659,6 @@
           <t>56</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>alto</t>

</xml_diff>

<commit_message>
Frequencia/volume/intensidade editaveis por aluno na aba Ciclo
- Frequencia: coluna frequencia (fallback = nº de dias de treino)
- Volume: total de series da semana, calculado do treino
- Intensidade: media de RPE da coluna rpe (mostra — se vazio)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -600,6 +600,21 @@
           <t>metas</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>frequencia</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>volume</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>intensidade</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -741,6 +756,11 @@
           <t>0</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -791,6 +811,11 @@
       <c r="J5" t="inlineStr">
         <is>
           <t>Agachamento sumô com 20 kg=60; Ganhar 500 g de massa muscular=0</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2x na semana + beach tênis</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona aluna Lara e melhorias na plataforma
- Nova aluna Lara (treinos A-E, foco emagrecimento/condicionamento)
- Etiquetas de metodo + legenda nos treinos (clareza pro aluno)
- Aba Evolucao: alunos sem avaliacao nao mostram mais dados de exemplo
- Atividades: remove termo tecnico MET da tela e adiciona Tenis,
  Beach tenis, CrossFit e Aula aerobica
- .gitignore protege fichas de anamnese (dados pessoais)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -819,6 +819,58 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Plano 3 meses</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Foco: emagrecimento e massa magra · Treinos A–E (seg a sex)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PERDA DE GORDURA E CONDICIONAMENTO</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Atleta experiente em musculação, em fase de retomada da constância. Objetivo principal: redução do percentual de gordura; meta secundária: aumento de massa magra. Periodização semanal de segunda a sexta, combinando musculação e corrida progressiva na esteira (método caminhada-corrida), com progressão gradual de volume e intensidade.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>5x na semana</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -830,7 +882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3239,6 +3291,1184 @@
       <c r="I55" t="inlineStr">
         <is>
           <t>Corpo alinhado, core contraído.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>A · Inferiores</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Agachamento cálice com halteres</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Pernas/glúteos · principal</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Método slow: diminuir a cadência na descida (descida lenta e controlada).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>A · Inferiores</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Cadeira extensora</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Quadríceps</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>15/12/10/08</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Progressão de carga: aumentar o peso a cada série.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>A · Inferiores</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Cadeira adutora</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Adutores</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>12 + 10s</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Faça 12 repetições e, ao terminar, segure 10 segundos de isometria (parada na contração) antes de descansar. Repita em todas as séries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>A · Inferiores</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Panturrilha em pé livre</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Panturrilha · tríceps sural</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>A · Inferiores</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Aeróbico leve — bicicleta</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Cardio · aeróbico</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>20 min</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Ritmo leve (intensidade baixa, respiração controlada).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>B · Superiores e Core</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Puxador frente com triângulo</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Dorsais · principal</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Pegada triângulo (delta). Puxar com os cotovelos, levando até o peito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>B · Superiores e Core</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Remada sentada na polia (pulley)</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Puxar próximo ao abdômen, peito aberto e coluna neutra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>B · Superiores e Core</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Supino sentada na máquina</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Peitoral</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Controlar a descida, sem travar os cotovelos no final.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>B · Superiores e Core</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Supino inclinado com halteres</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Peitoral superior</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Amplitude completa, sem bater os halteres no topo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>B · Superiores e Core</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Prancha abdominal</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>1 min</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Corpo alinhado da cabeça ao calcanhar, abdômen contraído.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>B · Superiores e Core</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Abdominal curto no solo</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Contraia o abdômen no topo, sem puxar o pescoço.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>B · Superiores e Core</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Aeróbico — caminhada na esteira</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Cardio · aeróbico</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>20 min</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Ritmo moderado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>C · Corrida + Braços/Ombros</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Esteira — aquecimento (caminhada)</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Cardio · aquecimento</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Caminhada leve (~5-6 km/h) para preparar o corpo. Respiração tranquila.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>C · Corrida + Braços/Ombros</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Esteira — blocos caminhada/corrida</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Cardio · intervalado</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>1 min corrida + 2 min caminhada</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Método caminhada-corrida (iniciante): a cada bloco, corra 1 min em ritmo leve (~7-8 km/h, dá pra falar frases curtas) e caminhe 2 min para recuperar (~5-6 km/h). Repita 4 blocos (~12 min). Progressão: quando ficar confortável, aumente a corrida para 2 min e/ou acrescente mais blocos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>C · Corrida + Braços/Ombros</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Esteira — desaquecimento (caminhada)</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Cardio · desaquecimento</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Caminhada leve diminuindo o ritmo aos poucos. Finalize com alongamento de pernas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>C · Corrida + Braços/Ombros</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Rosca direta com halteres</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Bíceps</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Cotovelos fixos junto ao corpo, sem balançar o tronco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>C · Corrida + Braços/Ombros</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Rosca martelo</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Bíceps · braquial</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Pegada neutra (palmas viradas uma para a outra). Subida controlada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>C · Corrida + Braços/Ombros</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Tríceps na polia com corda</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Tríceps</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Cotovelos fixos; abrir a corda no final do movimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>C · Corrida + Braços/Ombros</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Tríceps francês com halter</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Tríceps · cabeça longa</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Cotovelos apontando para cima, descer o peso atrás da cabeça com controle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>C · Corrida + Braços/Ombros</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Desenvolvimento com halteres</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Ombro · principal</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Core firme, sem arquear a lombar. Não travar os cotovelos no topo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>C · Corrida + Braços/Ombros</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Elevação lateral</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Deltoide medial</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Subir até a linha dos ombros, cotovelos levemente flexionados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>D · Posterior, Glúteos e Lombar</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Leg press</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Pernas</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Não estender totalmente os joelhos no topo; descida controlada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>D · Posterior, Glúteos e Lombar</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Cadeira flexora</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Movimento controlado, segurar 1s na contração.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>D · Posterior, Glúteos e Lombar</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Cadeira abdutora</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Glúteos · abdutores</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Abrir as pernas com controle, sem jogar o tronco para trás.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>D · Posterior, Glúteos e Lombar</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Cadeira romana (extensão lombar)</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Lombar · core</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Subir até alinhar o tronco; não hiperestender a lombar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>D · Posterior, Glúteos e Lombar</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Aeróbico — caminhada na esteira</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Cardio · aeróbico</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>20 min</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Ritmo moderado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>E · Corrida (Cardio)</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Esteira — aquecimento (caminhada)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Cardio · aquecimento</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Caminhada leve (~5-6 km/h) para preparar o corpo. Respiração tranquila.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>E · Corrida (Cardio)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Esteira — blocos caminhada/corrida</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Cardio · intervalado</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>1 min corrida + 2 min caminhada</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Método caminhada-corrida (iniciante): a cada bloco, corra 1 min em ritmo leve (~7-8 km/h, dá pra falar frases curtas) e caminhe 2 min para recuperar (~5-6 km/h). Repita 4 blocos (~12 min). Progressão: quando ficar confortável, aumente a corrida para 2 min e/ou acrescente mais blocos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>E · Corrida (Cardio)</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Esteira — desaquecimento (caminhada)</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Cardio · desaquecimento</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Caminhada leve diminuindo o ritmo aos poucos. Finalize com alongamento de pernas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige upload de foto (remove capture que forcava a camera) + padroniza notacao de drop set
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -871,6 +871,63 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Plano 3 meses</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Foco: perda de gordura e proporção · Musculação 4x + CrossFit</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>PERDA DE GORDURA E DEFINIÇÃO</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Objetivo: emagrecer e ganhar definição muscular. Rotina: SEG peito/ombro/tríceps · TER costas/bíceps · QUA manguito e estabilização · QUI quadríceps (presencial) · SEX CrossFit · SÁB pontos fracos · DOM atividade ao ar livre. Métodos: progressão de carga, drop set, bi-set e isometria.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Reduzir gordura corporal para 13%=0; Melhorar a proporção de massa muscular=0</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>4x musculação + CrossFit</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -882,7 +939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2127,7 +2184,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Drop set: reduzir a carga a cada parada.</t>
+          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2426,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Drop set: reduzir a carga a cada parada.</t>
+          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2747,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Drop set: reduzir a carga a cada parada.</t>
+          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -4469,6 +4526,1372 @@
       <c r="I84" t="inlineStr">
         <is>
           <t>Caminhada leve diminuindo o ritmo aos poucos. Finalize com alongamento de pernas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Supino inclinado com halteres</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Peitoral</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>15/12/10/08</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Progressão de carga ao longo das séries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Supino reto na máquina</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Peitoral</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>10 + 10</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>10 reps curtas + 10 completas em cada série.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Peck deck</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Peitoral</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>15/12/10</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Elevação lateral</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Deltóide lateral</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>15/12/10</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Elevação lateral no cabo</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Deltóide lateral</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Segura 1 seg no topo (isometria).</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Face pull</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Deltóide posterior</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Saúde do ombro: cotovelos altos, segura 1 seg na contração.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Tríceps barra reta no cross</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Tríceps</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>15/12/10</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Tríceps coice no cross</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Tríceps</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Trava o cotovelo, só o antebraço se move.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>B · Ter · Costas e Bíceps</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Puxada frente pegada aberta</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>20/15/12/10</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Progressão de carga ao longo das séries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>B · Ter · Costas e Bíceps</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Remada curvada ou na máquina</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>12/10/10/08</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Progressão de carga. Controla a fase negativa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>B · Ter · Costas e Bíceps</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Remada baixa / serrote</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>B · Ter · Costas e Bíceps</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Crucifixo inverso</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Deltóide posterior</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>B · Ter · Costas e Bíceps</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Rosca direta + rosca martelo (bi-set)</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Bíceps</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>12 cada</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Bi-set: as duas roscas em sequência, sem descanso entre elas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>B · Ter · Costas e Bíceps</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Rosca scott (banco)</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Bíceps</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>15/12/10</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>C · Qua · Manguito e Estabilização</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Rotação externa no cabo (cotovelo no corpo)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Manguito rotador</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>15 cada</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Cotovelo colado ao tronco, gira só o antebraço. Carga leve, controlada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>C · Qua · Manguito e Estabilização</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Rotação externa a 90° (cabo ou elástico)</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Manguito rotador</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>12 cada</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Braço a 90°: fortalece o manguito na posição de overhead do CrossFit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>C · Qua · Manguito e Estabilização</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Rotação interna no cabo</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Manguito rotador</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>15 cada</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Equilíbrio do manguito (subescapular).</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>C · Qua · Manguito e Estabilização</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Face pull</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Estabilizadores da escápula</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Retração escapular, cotovelos altos. Segura 1 seg na contração (isometria).</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>C · Qua · Manguito e Estabilização</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Y-T-W no banco inclinado</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Trapézio inferior/médio</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Movimentos lentos, polegar pra cima. Prehab escapular.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>C · Qua · Manguito e Estabilização</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Serrátil (serratus punch no cabo)</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Serrátil anterior</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Empurra e 'avança' a escápula no final do movimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>C · Qua · Manguito e Estabilização</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Pallof press no cabo</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Core · anti-rotação</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>12 cada</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Segura 2 seg na ponta (isometria anti-rotação). Tronco firme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>C · Qua · Manguito e Estabilização</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Prancha com toque no ombro</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Core · estabilização</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>20 toques</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Quadril estável, sem balançar. 20 toques no total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>D · Qui · Quadríceps</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Hack squat</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Quadríceps</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>15/12/10/08</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Progressão de carga. Único composto do dia — o agacho pesado já vem do CrossFit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>D · Qui · Quadríceps</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Cadeira extensora</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Quadríceps</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>15/12/10</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (15 → 12 → 10); segura 1 seg no topo de cada rep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>D · Qui · Quadríceps</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Mesa flexora</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>2 min de isometria ao final da última série.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>D · Qui · Quadríceps</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Cadeira adutora</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Adutores</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>15 ISO + 15</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>15 seg de isometria + 15 reps por série.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>D · Qui · Quadríceps</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Panturrilha em pé</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Panturrilha</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>20/15/12/12</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Progressão de carga. Amplitude total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>D · Qui · Quadríceps</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Panturrilha sentada</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Panturrilha</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>E · Sáb · Pontos Fracos</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Elevação lateral</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Deltóide lateral</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>20/15/12</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (20 → 15 → 12) até a falha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>E · Sáb · Pontos Fracos</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Rosca direta + tríceps na corda (bi-set)</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Bíceps/tríceps</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>15 cada</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Bi-set: um logo após o outro, sem descanso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>E · Sáb · Pontos Fracos</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Panturrilha em pé</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Panturrilha</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Segura 2 seg no topo (isometria).</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>E · Sáb · Pontos Fracos</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Abdominal na corda no pulley</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>E · Sáb · Pontos Fracos</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Prancha</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>40s</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Isometria: corpo alinhado, abdômen contraído.</t>
         </is>
       </c>
     </row>
@@ -4569,7 +5992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4920,6 +6343,307 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Composição</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Peso</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>83,6</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>83,6</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Composição</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>% Gordura</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>15,7</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>15,7</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Composição</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Massa magra</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>70,4</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>70,4</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Composição</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Gordura (kg)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>13,2</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>13,2</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Circunferências</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Cintura</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>85,4</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>85,4</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Circunferências</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Quadril</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>104,4</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>104,4</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Circunferências</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Braço (contraído)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>38,8</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>38,8</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>alto</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Circunferências</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Coxa medial</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>52,9</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>52,9</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>alto</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona aluna Lucila Mandirola (iniciante, ganho de massa, 2x musculacao + aerobica)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -834,6 +834,63 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Plano mensal</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Foco: ganho de massa · Iniciante · Musculação 2x + aulas aeróbicas</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ADAPTAÇÃO E GANHO DE MASSA</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Objetivo: ganho de massa muscular. Iniciante na musculação, construindo base, técnica e constância. Rotina: SEG aula aeróbica · TER pernas completas (presencial) · QUA aula aeróbica · QUI aula aeróbica · SEX superiores (presencial). Foco em execução correta e progressão gradual de carga semana a semana.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Dominar a técnica dos exercícios base=0; Criar constância: não faltar nos treinos da semana=0</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2x musculação + aulas aeróbicas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -845,7 +902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4742,6 +4799,700 @@
       <c r="I95" t="inlineStr">
         <is>
           <t>Isometria: corpo alinhado, abdômen contraído.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>A · Terça · Pernas completas</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Aquecimento · 8 min de bike ou esteira</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Aquecimento</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>8 min</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Ritmo leve, só pra aquecer e soltar o corpo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>A · Terça · Pernas completas</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Leg press 45°</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Quadríceps/glúteos</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>12-15</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Desce controlado até uns 90°, sem tirar o quadril do banco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>A · Terça · Pernas completas</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Cadeira extensora</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Quadríceps</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>12-15</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Segura 1 seg no topo, descida controlada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>A · Terça · Pernas completas</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Mesa flexora</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Posterior de coxa</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>12-15</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Sem usar impulso, foco no posterior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>A · Terça · Pernas completas</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Elevação pélvica (hip thrust)</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Glúteos</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Aperta o glúteo lá no topo do movimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>A · Terça · Pernas completas</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Cadeira abdutora</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Glúteo médio</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>A · Terça · Pernas completas</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Cadeira adutora</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Adutores</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>A · Terça · Pernas completas</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Panturrilha em pé</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Panturrilha</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>15-20</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Amplitude total: alonga embaixo, sobe no talão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>B · Sexta · Superiores</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Aquecimento · 5 min de bike ou elíptico</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Aquecimento</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Ritmo leve pra aquecer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>B · Sexta · Superiores</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Supino na máquina (ou halteres)</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Peitoral</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>12-15</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Cotovelos a ~45°, desce controlado até a linha do peito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>B · Sexta · Superiores</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Puxada frente (pulldown)</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>12-15</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Puxa com os cotovelos, peito aberto, sem balançar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>B · Sexta · Superiores</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Remada na máquina</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>12-15</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Aproxima as escápulas no fim do movimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>B · Sexta · Superiores</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Desenvolvimento na máquina</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Ombro</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Não estende o cotovelo até travar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>B · Sexta · Superiores</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Elevação lateral</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Deltóide lateral</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>12-15</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Carga leve, sobe até a linha do ombro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>B · Sexta · Superiores</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Rosca direta</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Bíceps</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Cotovelo parado junto ao corpo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>B · Sexta · Superiores</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Tríceps na corda (pulley)</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Tríceps</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>12-15</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Estende o cotovelo até embaixo, controla a volta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>B · Sexta · Superiores</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Abdominal</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Contrai o abdômen, sem puxar o pescoço.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajusta treino do Nilo: dia C (manguito) e dia E (pontos fracos)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -902,7 +902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J112"/>
+  <dimension ref="A1:J116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3439,7 +3439,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3449,39 +3449,34 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>A · Seg · Peito, Ombro e Tríceps</t>
+          <t>A · Terça · Pernas completas</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Supino inclinado com halteres</t>
+          <t>Aquecimento · 8 min de bike ou esteira</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Peitoral</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>4</t>
+          <t>Aquecimento</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>15/12/10/08</t>
+          <t>8 min</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Progressão de carga ao longo das séries.</t>
+          <t>Ritmo leve, só pra aquecer e soltar o corpo.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3491,39 +3486,39 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>A · Seg · Peito, Ombro e Tríceps</t>
+          <t>A · Terça · Pernas completas</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Supino reto na máquina</t>
+          <t>Leg press 45°</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Peitoral</t>
+          <t>Quadríceps/glúteos</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>10 + 10</t>
+          <t>12-15</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>10 reps curtas + 10 completas em cada série.</t>
+          <t>Desce controlado até uns 90°, sem tirar o quadril do banco.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3533,17 +3528,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>A · Seg · Peito, Ombro e Tríceps</t>
+          <t>A · Terça · Pernas completas</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Peck deck</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Peitoral</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3553,19 +3548,19 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>12-15</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Segura 1 seg no topo, descida controlada.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3575,39 +3570,39 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>A · Seg · Peito, Ombro e Tríceps</t>
+          <t>A · Terça · Pernas completas</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Elevação lateral</t>
+          <t>Mesa flexora</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Deltóide lateral</t>
+          <t>Posterior de coxa</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>12-15</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Sem usar impulso, foco no posterior.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3617,17 +3612,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>A · Seg · Peito, Ombro e Tríceps</t>
+          <t>A · Terça · Pernas completas</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Elevação lateral no cabo</t>
+          <t>Elevação pélvica (hip thrust)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Deltóide lateral</t>
+          <t>Glúteos</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3637,19 +3632,19 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Segura 1 seg no topo (isometria).</t>
+          <t>Aperta o glúteo lá no topo do movimento.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3659,17 +3654,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>A · Seg · Peito, Ombro e Tríceps</t>
+          <t>A · Terça · Pernas completas</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Face pull</t>
+          <t>Cadeira abdutora</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Deltóide posterior</t>
+          <t>Glúteo médio</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3680,18 +3675,13 @@
       <c r="G68" t="inlineStr">
         <is>
           <t>15</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>Saúde do ombro: cotovelos altos, segura 1 seg na contração.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3701,17 +3691,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>A · Seg · Peito, Ombro e Tríceps</t>
+          <t>A · Terça · Pernas completas</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Tríceps barra reta no cross</t>
+          <t>Cadeira adutora</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Tríceps</t>
+          <t>Adutores</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3721,19 +3711,14 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>15/12/10</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3743,39 +3728,39 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>A · Seg · Peito, Ombro e Tríceps</t>
+          <t>A · Terça · Pernas completas</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Tríceps coice no cross</t>
+          <t>Panturrilha em pé</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Tríceps</t>
+          <t>Panturrilha</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15-20</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Trava o cotovelo, só o antebraço se move.</t>
+          <t>Amplitude total: alonga embaixo, sobe no talão.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3785,39 +3770,34 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>B · Ter · Costas e Bíceps</t>
+          <t>B · Sexta · Superiores</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Puxada frente pegada aberta</t>
+          <t>Aquecimento · 5 min de bike ou elíptico</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Costas</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>4</t>
+          <t>Aquecimento</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>20/15/12/10</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Progressão de carga ao longo das séries.</t>
+          <t>Ritmo leve pra aquecer.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3827,39 +3807,39 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>B · Ter · Costas e Bíceps</t>
+          <t>B · Sexta · Superiores</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Remada curvada ou na máquina</t>
+          <t>Supino na máquina (ou halteres)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Peitoral</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>12/10/10/08</t>
+          <t>12-15</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Progressão de carga. Controla a fase negativa.</t>
+          <t>Cotovelos a ~45°, desce controlado até a linha do peito.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3869,12 +3849,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>B · Ter · Costas e Bíceps</t>
+          <t>B · Sexta · Superiores</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Remada baixa / serrote</t>
+          <t>Puxada frente (pulldown)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3889,14 +3869,19 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12-15</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Puxa com os cotovelos, peito aberto, sem balançar.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3906,17 +3891,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>B · Ter · Costas e Bíceps</t>
+          <t>B · Sexta · Superiores</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Crucifixo inverso</t>
+          <t>Remada na máquina</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Deltóide posterior</t>
+          <t>Costas</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3926,14 +3911,19 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12-15</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Aproxima as escápulas no fim do movimento.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3943,39 +3933,39 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>B · Ter · Costas e Bíceps</t>
+          <t>B · Sexta · Superiores</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Rosca direta + rosca martelo (bi-set)</t>
+          <t>Desenvolvimento na máquina</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Bíceps</t>
+          <t>Ombro</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>12 cada</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Bi-set: as duas roscas em sequência, sem descanso entre elas.</t>
+          <t>Não estende o cotovelo até travar.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3985,17 +3975,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>B · Ter · Costas e Bíceps</t>
+          <t>B · Sexta · Superiores</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Rosca scott (banco)</t>
+          <t>Elevação lateral</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Bíceps</t>
+          <t>Deltóide lateral</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -4005,39 +3995,39 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>12-15</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Carga leve, sobe até a linha do ombro.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>C · Qua · Manguito e Estabilização</t>
+          <t>B · Sexta · Superiores</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Rotação externa no cabo (cotovelo no corpo)</t>
+          <t>Rosca direta</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Manguito rotador</t>
+          <t>Bíceps</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -4047,39 +4037,39 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>15 cada</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Cotovelo colado ao tronco, gira só o antebraço. Carga leve, controlada.</t>
+          <t>Cotovelo parado junto ao corpo.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>C · Qua · Manguito e Estabilização</t>
+          <t>B · Sexta · Superiores</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Rotação externa a 90° (cabo ou elástico)</t>
+          <t>Tríceps na corda (pulley)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Manguito rotador</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -4089,39 +4079,39 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>12 cada</t>
+          <t>12-15</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Braço a 90°: fortalece o manguito na posição de overhead do CrossFit.</t>
+          <t>Estende o cotovelo até embaixo, controla a volta.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Nilo Sheeny</t>
+          <t>Lucila Mandirola</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>C · Qua · Manguito e Estabilização</t>
+          <t>B · Sexta · Superiores</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Rotação interna no cabo</t>
+          <t>Abdominal</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Manguito rotador</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -4131,12 +4121,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>15 cada</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Equilíbrio do manguito (subescapular).</t>
+          <t>Contrai o abdômen, sem puxar o pescoço.</t>
         </is>
       </c>
     </row>
@@ -4148,37 +4138,37 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>C · Qua · Manguito e Estabilização</t>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Face pull</t>
+          <t>Supino inclinado com halteres</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Estabilizadores da escápula</t>
+          <t>Peitoral</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15/12/10/08</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Retração escapular, cotovelos altos. Segura 1 seg na contração (isometria).</t>
+          <t>Progressão de carga ao longo das séries.</t>
         </is>
       </c>
     </row>
@@ -4190,37 +4180,37 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>C · Qua · Manguito e Estabilização</t>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Y-T-W no banco inclinado</t>
+          <t>Supino reto na máquina</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Trapézio inferior/médio</t>
+          <t>Peitoral</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10 + 10</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Movimentos lentos, polegar pra cima. Prehab escapular.</t>
+          <t>10 reps curtas + 10 completas em cada série.</t>
         </is>
       </c>
     </row>
@@ -4232,22 +4222,22 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>C · Qua · Manguito e Estabilização</t>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Serrátil (serratus punch no cabo)</t>
+          <t>Peck deck</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Serrátil anterior</t>
+          <t>Peitoral</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -4257,12 +4247,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Empurra e 'avança' a escápula no final do movimento.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -4274,37 +4264,37 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>C · Qua · Manguito e Estabilização</t>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Pallof press no cabo</t>
+          <t>Elevação lateral</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Core · anti-rotação</t>
+          <t>Deltóide lateral</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>12 cada</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Segura 2 seg na ponta (isometria anti-rotação). Tronco firme.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -4316,22 +4306,22 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>C · Qua · Manguito e Estabilização</t>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Prancha com toque no ombro</t>
+          <t>Elevação lateral no cabo</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Core · estabilização</t>
+          <t>Deltóide lateral</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -4341,12 +4331,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>20 toques</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Quadril estável, sem balançar. 20 toques no total.</t>
+          <t>Segura 1 seg no topo (isometria).</t>
         </is>
       </c>
     </row>
@@ -4358,37 +4348,37 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>D · Qui · Quadríceps</t>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Hack squat</t>
+          <t>Face pull</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Deltóide posterior</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>15/12/10/08</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Progressão de carga. Único composto do dia — o agacho pesado já vem do CrossFit.</t>
+          <t>Saúde do ombro: cotovelos altos, segura 1 seg na contração.</t>
         </is>
       </c>
     </row>
@@ -4400,27 +4390,27 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>D · Qui · Quadríceps</t>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Cadeira extensora</t>
+          <t>Tríceps barra reta no cross</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4430,7 +4420,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (15 → 12 → 10); segura 1 seg no topo de cada rep.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -4442,27 +4432,27 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>D · Qui · Quadríceps</t>
+          <t>A · Seg · Peito, Ombro e Tríceps</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Mesa flexora</t>
+          <t>Tríceps coice no cross</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -4472,7 +4462,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2 min de isometria ao final da última série.</t>
+          <t>Trava o cotovelo, só o antebraço se move.</t>
         </is>
       </c>
     </row>
@@ -4484,37 +4474,37 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>D · Qui · Quadríceps</t>
+          <t>B · Ter · Costas e Bíceps</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Cadeira adutora</t>
+          <t>Puxada frente pegada aberta</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Adutores</t>
+          <t>Costas</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>15 ISO + 15</t>
+          <t>20/15/12/10</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>15 seg de isometria + 15 reps por série.</t>
+          <t>Progressão de carga ao longo das séries.</t>
         </is>
       </c>
     </row>
@@ -4526,22 +4516,22 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>D · Qui · Quadríceps</t>
+          <t>B · Ter · Costas e Bíceps</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Panturrilha em pé</t>
+          <t>Remada curvada ou na máquina</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Panturrilha</t>
+          <t>Costas</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4551,12 +4541,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>20/15/12/12</t>
+          <t>12/10/10/08</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Progressão de carga. Amplitude total.</t>
+          <t>Progressão de carga. Controla a fase negativa.</t>
         </is>
       </c>
     </row>
@@ -4568,22 +4558,22 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>D · Qui · Quadríceps</t>
+          <t>B · Ter · Costas e Bíceps</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Panturrilha sentada</t>
+          <t>Remada baixa / serrote</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Panturrilha</t>
+          <t>Costas</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -4593,7 +4583,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -4605,37 +4595,32 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>E · Sáb · Pontos Fracos</t>
+          <t>B · Ter · Costas e Bíceps</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Elevação lateral</t>
+          <t>Crucifixo inverso</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Deltóide lateral</t>
+          <t>Deltóide posterior</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>20/15/12</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>Drop set: tudo na MESMA série — reduz a carga sem descanso (20 → 15 → 12) até a falha.</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -4647,37 +4632,37 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>E · Sáb · Pontos Fracos</t>
+          <t>B · Ter · Costas e Bíceps</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Rosca direta + tríceps na corda (bi-set)</t>
+          <t>Rosca direta + rosca martelo (bi-set)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Bíceps/tríceps</t>
+          <t>Bíceps</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>15 cada</t>
+          <t>12 cada</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Bi-set: um logo após o outro, sem descanso.</t>
+          <t>Bi-set: as duas roscas em sequência, sem descanso entre elas.</t>
         </is>
       </c>
     </row>
@@ -4689,22 +4674,22 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>E · Sáb · Pontos Fracos</t>
+          <t>B · Ter · Costas e Bíceps</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Panturrilha em pé</t>
+          <t>Rosca scott (banco)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Panturrilha</t>
+          <t>Bíceps</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -4714,12 +4699,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Segura 2 seg no topo (isometria).</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -4731,22 +4716,22 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>E · Sáb · Pontos Fracos</t>
+          <t>C · Qua · Manguito e Estabilização</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Abdominal na corda no pulley</t>
+          <t>Rotação externa a 90° (cabo ou elástico)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Manguito rotador</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4756,7 +4741,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12 cada</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Braço a 90°: fortalece o manguito na posição de overhead do CrossFit.</t>
         </is>
       </c>
     </row>
@@ -4768,22 +4758,22 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>E · Sáb · Pontos Fracos</t>
+          <t>C · Qua · Manguito e Estabilização</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Prancha</t>
+          <t>Rotação interna no cabo</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Manguito rotador</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4793,76 +4783,81 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>40s</t>
+          <t>15 cada</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Isometria: corpo alinhado, abdômen contraído.</t>
+          <t>Equilíbrio do manguito (subescapular).</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>A · Terça · Pernas completas</t>
+          <t>C · Qua · Manguito e Estabilização</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Aquecimento · 8 min de bike ou esteira</t>
+          <t>Face pull</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Aquecimento</t>
+          <t>Estabilizadores da escápula</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>8 min</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>Ritmo leve, só pra aquecer e soltar o corpo.</t>
+          <t>Retração escapular, cotovelos altos. Segura 1 seg na contração (isometria).</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>A · Terça · Pernas completas</t>
+          <t>C · Qua · Manguito e Estabilização</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Leg press 45°</t>
+          <t>Band pull-apart (abertura com elástico)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Quadríceps/glúteos</t>
+          <t>Trapézio médio/posterior</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -4872,39 +4867,39 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>12-15</t>
+          <t>15-20</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>Desce controlado até uns 90°, sem tirar o quadril do banco.</t>
+          <t>Abre o elástico à frente do corpo juntando as escápulas. Prehab de ombro, carga leve.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>A · Terça · Pernas completas</t>
+          <t>C · Qua · Manguito e Estabilização</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Cadeira extensora</t>
+          <t>Serrátil (serratus punch no cabo)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Serrátil anterior</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4914,39 +4909,39 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>12-15</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Segura 1 seg no topo, descida controlada.</t>
+          <t>Empurra e 'avança' a escápula no final do movimento.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>A · Terça · Pernas completas</t>
+          <t>C · Qua · Manguito e Estabilização</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Mesa flexora</t>
+          <t>Pallof press no cabo</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Posterior de coxa</t>
+          <t>Core · anti-rotação</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -4956,39 +4951,39 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>12-15</t>
+          <t>12 cada</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Sem usar impulso, foco no posterior.</t>
+          <t>Segura 2 seg na ponta (isometria anti-rotação). Tronco firme.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>A · Terça · Pernas completas</t>
+          <t>C · Qua · Manguito e Estabilização</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Elevação pélvica (hip thrust)</t>
+          <t>Prancha com toque no ombro</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Glúteos</t>
+          <t>Core · estabilização</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -4998,113 +4993,123 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>20 toques</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Aperta o glúteo lá no topo do movimento.</t>
+          <t>Quadril estável, sem balançar. 20 toques no total.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>A · Terça · Pernas completas</t>
+          <t>D · Qui · Quadríceps</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Cadeira abdutora</t>
+          <t>Hack squat</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Glúteo médio</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15/12/10/08</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Progressão de carga. Único composto do dia (o agacho pesado já vem do CrossFit).</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>A · Terça · Pernas completas</t>
+          <t>D · Qui · Quadríceps</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Cadeira adutora</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Adutores</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15/12/10</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso; segura 1 seg no topo de cada rep.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>A · Terça · Pernas completas</t>
+          <t>D · Qui · Quadríceps</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Panturrilha em pé</t>
+          <t>Mesa flexora</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Panturrilha</t>
+          <t>Posterior</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -5114,118 +5119,123 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>15-20</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Amplitude total: alonga embaixo, sobe no talão.</t>
+          <t>2 min de isometria ao final da última série.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>B · Sexta · Superiores</t>
+          <t>D · Qui · Quadríceps</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Aquecimento · 5 min de bike ou elíptico</t>
+          <t>Cadeira adutora</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Aquecimento</t>
+          <t>Adutores</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>15 ISO + 15</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Ritmo leve pra aquecer.</t>
+          <t>15 seg de isometria + 15 reps por série.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>B · Sexta · Superiores</t>
+          <t>D · Qui · Quadríceps</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Supino na máquina (ou halteres)</t>
+          <t>Panturrilha em pé</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Peitoral</t>
+          <t>Panturrilha</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>12-15</t>
+          <t>20/15/12/12</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Cotovelos a ~45°, desce controlado até a linha do peito.</t>
+          <t>Progressão de carga. Amplitude total.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>B · Sexta · Superiores</t>
+          <t>D · Qui · Quadríceps</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Puxada frente (pulldown)</t>
+          <t>Panturrilha sentada</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Panturrilha</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -5235,81 +5245,76 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>12-15</t>
-        </is>
-      </c>
-      <c r="I106" t="inlineStr">
-        <is>
-          <t>Puxa com os cotovelos, peito aberto, sem balançar.</t>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>B · Sexta · Superiores</t>
+          <t>E · Sáb · Pontos Fracos</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Remada na máquina</t>
+          <t>Elevação lateral</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Deltóide lateral</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>12-15</t>
+          <t>20/15/12</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Aproxima as escápulas no fim do movimento.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (20 → 15 → 12) até a falha.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>B · Sexta · Superiores</t>
+          <t>E · Sáb · Pontos Fracos</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Desenvolvimento na máquina</t>
+          <t>Elevação lateral no cabo (unilateral)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Ombro</t>
+          <t>Deltóide lateral</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -5319,39 +5324,39 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>Não estende o cotovelo até travar.</t>
+          <t>Carga leve, um braço de cada vez, controla a descida.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>B · Sexta · Superiores</t>
+          <t>E · Sáb · Pontos Fracos</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Elevação lateral</t>
+          <t>Crucifixo inverso</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Deltóide lateral</t>
+          <t>Deltóide posterior</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -5361,39 +5366,39 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>12-15</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Carga leve, sobe até a linha do ombro.</t>
+          <t>Ombro posterior: aperta as escápulas no fim do movimento.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>B · Sexta · Superiores</t>
+          <t>E · Sáb · Pontos Fracos</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Rosca direta</t>
+          <t>Rosca direta + tríceps na corda (bi-set)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Bíceps</t>
+          <t>Bíceps/tríceps</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -5403,39 +5408,39 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15 cada</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Cotovelo parado junto ao corpo.</t>
+          <t>Bi-set: um logo após o outro, sem descanso.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>B · Sexta · Superiores</t>
+          <t>E · Sáb · Pontos Fracos</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Tríceps na corda (pulley)</t>
+          <t>Rosca martelo</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Tríceps</t>
+          <t>Bíceps</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -5445,54 +5450,212 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>12-15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Estende o cotovelo até embaixo, controla a volta.</t>
+          <t>Pegada neutra, cotovelo fixo junto ao corpo.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Lucila Mandirola</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>B · Sexta · Superiores</t>
+          <t>E · Sáb · Pontos Fracos</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Abdominal</t>
+          <t>Tríceps testa</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
+          <t>Tríceps</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Cotovelos apontados pra frente, controla a descida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>E · Sáb · Pontos Fracos</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Panturrilha em pé</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Panturrilha</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Segura 2 seg no topo (isometria).</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>E · Sáb · Pontos Fracos</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Panturrilha sentada</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Panturrilha</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>E · Sáb · Pontos Fracos</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Abdominal na corda no pulley</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
           <t>Core</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr">
+      <c r="F115" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr">
+      <c r="G115" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>Contrai o abdômen, sem puxar o pescoço.</t>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>E · Sáb · Pontos Fracos</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Prancha</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>40s</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Isometria: corpo alinhado, abdômen contraído.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Macrociclo personalizado por aluno (aba Periodizacao) + periodizacao do Nilo + novo objetivo
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Treinos" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Biblioteca" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Avaliacao" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Periodizacao" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -535,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -615,6 +616,11 @@
           <t>intensidade</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ciclo_semana</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -800,7 +806,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Objetivo: emagrecer e ganhar definição muscular. Rotina: SEG peito/ombro/tríceps · TER costas/bíceps · QUA manguito e estabilização · QUI quadríceps (presencial) · SEX CrossFit · SÁB pontos fracos · DOM atividade ao ar livre. Métodos: progressão de carga, drop set, bi-set e isometria.</t>
+          <t>Foco em recomposição: reduzir o percentual de gordura sem perder massa, melhorando a proporção e a definição. Como atleta avançado, une a musculação ao CrossFit num ciclo de 12 semanas que começa corrigindo limitações funcionais, passa pela hipertrofia dos pontos fracos e fecha na definição. O que conta aqui é constância, técnica impecável e recuperação de qualidade.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -832,6 +838,9 @@
         <is>
           <t>4x musculação + CrossFit</t>
         </is>
+      </c>
+      <c r="N5" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -6411,4 +6420,240 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>aluno</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>bloco</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>foco</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>descricao</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>semanas</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>intensidade</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bloco 1 · Adaptação e Correção</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CORREÇÃO E BASE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Técnica, prehab de ombro e quadril, correção de assimetrias. Cargas controladas.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Semanas 1–3</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>RPE 6–7</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>concluido</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bloco 2 · Hipertrofia</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>VOLUME E PROPORÇÃO</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Volume alto nos pontos fracos (ombro, braço, peito, panturrilha). Drop set e bi-set.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Semanas 4–7</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>RPE 7–8</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>agora</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Deload</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>RECUPERAÇÃO</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Semana leve para recuperar e supercompensar. A folga faz parte do resultado.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Semana 8</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>RPE 5–6</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bloco 3 · Definição</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DENSIDADE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Manter o músculo no déficit: composto mais pesado e finalizadores metabólicos. O CrossFit puxa o gasto.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Semanas 9–11</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>RPE 8</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Nilo Sheeny</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bloco 4 · Reavaliação</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>AJUSTE</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Pico de definição, reavaliação do percentual de gordura e plano do próximo ciclo.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Semana 12</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>RPE 7 → leve</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Periodizacao (macrociclo) personalizada para todas as alunas
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -673,6 +673,9 @@
           <t>5</t>
         </is>
       </c>
+      <c r="N2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -730,6 +733,9 @@
           <t>2x na semana + beach tênis</t>
         </is>
       </c>
+      <c r="N3" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -782,6 +788,9 @@
           <t>5x na semana</t>
         </is>
       </c>
+      <c r="N4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -898,6 +907,9 @@
         <is>
           <t>2x musculação + aulas aeróbicas</t>
         </is>
+      </c>
+      <c r="N6" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -6428,7 +6440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6653,6 +6665,635 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Bloco 1 · Adaptação</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BASE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Reconexão e técnica, retomando o volume de treino.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Semanas 1–2</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>RPE 6–7</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>concluido</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bloco 2 · Acúmulo</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>HIPERTROFIA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Volume alto e progressão de carga, foco em inferiores e glúteos.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Semanas 3–6</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>RPE 7–8</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>agora</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Deload</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>RECUPERAÇÃO</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Semana leve para recuperar e supercompensar.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Semana 7</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>RPE 5–6</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bloco 3 · Intensificação</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>FORÇA + MASSA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Cargas mais altas para ganhar força e estimular o ganho de massa.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Semanas 8–11</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>RPE 8–9</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Bloco 4 · Reavaliação</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>AJUSTE</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Checagem das metas do trimestre (agachamento sumô 20 kg, +500 g de massa) e novo ciclo.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Semana 12</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>RPE leve</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Bloco 1 · Retomada</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CONSTÂNCIA E BASE</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Reconstruir a constância e a técnica. Corrida no método caminhada-corrida.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Semanas 1–3</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>RPE 6–7</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>agora</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Bloco 2 · Hipertrofia metabólica</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MASSA + GASTO</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Volume para preservar massa magra e densidade para o gasto calórico. Corrida progride.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Semanas 4–7</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>RPE 7–8</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Deload</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>RECUPERAÇÃO</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Semana leve para recuperar.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Semana 8</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>RPE 5–6</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Bloco 3 · Definição</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>DENSIDADE</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Manter o músculo no déficit, corrida mais intensa.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Semanas 9–11</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>RPE 8</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Bloco 4 · Reavaliação</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>AJUSTE</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Reavaliação do percentual de gordura e ajustes do próximo ciclo.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Semana 12</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>RPE leve</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Karen Amor</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bloco 1 · Adaptação</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>RETORNO SEGURO</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Voltar a treinar com segurança: técnica e cargas leves, criar o hábito. Corrida quarta e domingo.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Semanas 1–4</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>RPE 5–6</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>agora</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Karen Amor</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Bloco 2 · Condicionamento</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BASE AERÓBICA</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Aumentar o volume e o condicionamento físico e respiratório, progressão da corrida.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Semanas 5–12</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>RPE 6–7</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Karen Amor</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Deload</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>RECUPERAÇÃO</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Semana leve para recuperar.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Semana 13</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>RPE 5</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Karen Amor</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Bloco 3 · Progressão</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CARGA E RESISTÊNCIA</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Progressão de carga e de resistência, consolidando o condicionamento.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Semanas 14–22</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>RPE 7–8</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Karen Amor</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Bloco 4 · Reavaliação</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>AJUSTE</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Reavaliação e plano do próximo ciclo.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Semanas 23–24</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>RPE leve</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Bloco 1 · Adaptação</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TÉCNICA E HÁBITO</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Aprender a execução dos exercícios e criar o hábito. Cargas leves e controladas.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Semanas 1–2</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>RPE 5–6</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>agora</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Lucila Mandirola</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Bloco 2 · Progressão inicial</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>PROGRESSÃO</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Subir a carga aos poucos mantendo a técnica impecável.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Semanas 3–4</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>RPE 6–7</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona aluno Felipe (musculacao 3x + corrida) e campo de tempo no cardio
- Novo app do Felipe: peito/costas/pernas + corrida progressiva no sabado
- Sabado em blocos por semana, cada um com registro de tempo
- Cardio (corrida) agora registra tempo em vez de carga (corrige Karen e Lara)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -912,6 +912,66 @@
         <v>1</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Plano 3 meses</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Foco: peito, costas e pernas · Musculação 3x + CrossFit + corrida</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>HIPERTROFIA E INÍCIO DE CORRIDA</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Foco em hipertrofia de peito, costas e pernas, com três dias de musculação que complementam o CrossFit de segunda e quarta, sem repetir a sobrecarga de coluna dos WODs. No sábado entra a iniciação à corrida, em base aeróbica (Z2) com progressão de volume, respeitando a recuperação. O que conta aqui é constância, técnica impecável e progressão de carga semana a semana.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>23/07/2026</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Correr 5 km contínuos sem parar=0; Ganhar massa em peito, costas e pernas=0</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>3x musculação + CrossFit + corrida</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -923,7 +983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J116"/>
+  <dimension ref="A1:J142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5677,6 +5737,1078 @@
       <c r="I116" t="inlineStr">
         <is>
           <t>Isometria: corpo alinhado, abdômen contraído.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>A · Ter · Peito</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Supino na máquina (chest press)</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Peitoral · principal</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>12/10/8/8</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Progressão de carga ao longo das séries. Empurra controlado, sem travar o cotovelo no fim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>A · Ter · Peito</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Supino inclinado com halteres</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Peitoral</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Progressão de carga: aumente o peso a cada série mantendo a técnica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>A · Ter · Peito</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Crucifixo na máquina (voador)</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Peitoral</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Abre bem e segura 1 seg na contração.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>A · Ter · Peito</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Crossover na polia</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Peitoral</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>15/12/10</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>A · Ter · Peito</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Tríceps na corda</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Tríceps</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Cotovelos fixos junto ao corpo, abre bem no fim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>A · Ter · Peito</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Tríceps testa</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Tríceps</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>15/12/10</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>B · Qui · Costas</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Barra fixa ou puxada alta (pegada aberta)</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Costas · principal</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>12/10/8/8</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Progressão de carga ao longo das séries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>B · Qui · Costas</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Remada sentada na máquina (pegada neutra)</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>12/10/10/08</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Progressão de carga. Controla a fase negativa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>B · Qui · Costas</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Remada cavalinho (T-bar)</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>10-12</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Peito apoiado, puxa com os cotovelos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>B · Qui · Costas</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Puxada com triângulo (pegada neutra)</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Leva o triângulo ao peito, escápulas pra baixo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>B · Qui · Costas</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Pullover na polia</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Sente o dorsal alongar e contrair, cotovelos semi-fixos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>B · Qui · Costas</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Remada unilateral com halter (serrote)</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Costas</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>10 cada</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Um lado de cada vez, sem rodar o tronco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>B · Qui · Costas</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Rosca scott (banco)</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Bíceps</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>10-12</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Progressão de carga: aumente o peso a cada série. Cotovelos apoiados no banco, sobe e desce controlado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>C · Sex · Pernas</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Leg press 45°</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Pernas · principal</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>12/10/10/08</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Progressão de carga. Pés na largura do quadril, desce controlado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>C · Sex · Pernas</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Agachamento hack</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Quadríceps</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>10-12</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Máquina, poupando a coluna que o CrossFit já castiga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>C · Sex · Pernas</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Cadeira extensora</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Quadríceps</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>15/12/10</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>C · Sex · Pernas</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Mesa flexora (posterior)</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>12/10/10/10</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Progressão de carga. Controla a fase negativa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>C · Sex · Pernas</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Coice de glúteo na polia</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Glúteos</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>12 cada</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Um lado de cada vez, segura 1 seg na contração do glúteo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>C · Sex · Pernas</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Elevação pélvica (glúteo)</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Glúteos</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Segura 2 seg no topo (isometria) apertando o glúteo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>C · Sex · Pernas</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Panturrilha em pé</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Panturrilha</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>20/15/12/12</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Drop set na última série + isometria de 2 seg no topo de cada rep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>D · Sáb · Corrida</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Aquecimento</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Corrida · aquecimento</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Faça o aquecimento, depois SÓ o bloco da semana atual do seu ciclo, e termine no desaquecimento. A cada 4 semanas o ciclo recomeça, subindo cerca de 10%. Comece com caminhada rápida evoluindo para trote leve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>D · Sáb · Corrida</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Semana 1 · Corrida contínua leve</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Corrida · Semana 1</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>4-5 km</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Ritmo de conversa (Z2): você consegue falar frases inteiras. Registre seu tempo total no fim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>D · Sáb · Corrida</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Semana 2 · Fartlek</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Corrida · Semana 2</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>(3 min corrida + 1 min caminhada)</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>6 blocos de 3 min correndo moderado + 1 min caminhando. Registre o tempo total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>D · Sáb · Corrida</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Semana 3 · Longão leve</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Corrida · Semana 3</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr"/>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>5-6 km</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Contínuo em Z2, sem pressa, construindo resistência. Registre seu tempo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>D · Sáb · Corrida</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Semana 4 · Progressiva</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Corrida · Semana 4</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>5 km</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Comece leve e termine o último km mais forte (limiar leve). Registre seu tempo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>D · Sáb · Corrida</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Desaquecimento</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Corrida · volta à calma</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Trote bem leve até virar caminhada, depois alongue panturrilha, posterior e quadril.</t>
         </is>
       </c>
     </row>
@@ -6440,7 +7572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7294,6 +8426,191 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Bloco 1 · Adaptação</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BASE E TÉCNICA</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Execução perfeita, ativação de peito, costas e pernas e início da corrida leve no sábado. Cargas controladas.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Semanas 1–3</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>RPE 6–7</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>agora</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Bloco 2 · Hipertrofia</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>VOLUME</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Mais volume em peito, costas e pernas, com progressão de carga e drop sets. A corrida sobe de distância.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Semanas 4–7</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>RPE 7–8</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Deload</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>RECUPERAÇÃO</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Semana leve para recuperar e supercompensar. A folga faz parte do resultado.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Semana 8</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>RPE 5–6</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Bloco 3 · Força e Densidade</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CARGA</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Cargas mais altas nos compostos, mantendo a corrida em base aeróbica. Músculo mais denso e forte.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Semanas 9–11</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>RPE 8</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Bloco 4 · Reavaliação</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>AJUSTE</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Reavaliação física e teste de 5 km contínuos. Plano do próximo ciclo.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Semana 12</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>RPE 7 → leve</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>futuro</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refina objetivo do Felipe (perda de gordura como foco principal)
Objetivo: perda de gordura; musculacao pra ganhar musculo e complementar o
CrossFit; corrida e condicionamento como atividade extra.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -925,17 +925,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Foco: peito, costas e pernas · Musculação 3x + CrossFit + corrida</t>
+          <t>Foco: perda de gordura e ganho muscular · Musculação 3x + CrossFit + corrida</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>HIPERTROFIA E INÍCIO DE CORRIDA</t>
+          <t>PERDA DE GORDURA E GANHO MUSCULAR</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Foco em hipertrofia de peito, costas e pernas, com três dias de musculação que complementam o CrossFit de segunda e quarta, sem repetir a sobrecarga de coluna dos WODs. No sábado entra a iniciação à corrida, em base aeróbica (Z2) com progressão de volume, respeitando a recuperação. O que conta aqui é constância, técnica impecável e progressão de carga semana a semana.</t>
+          <t>O objetivo principal do Felipe é reduzir o percentual de gordura. A musculação, em três dias (peito, costas e pernas), entra pra ganhar mais músculo e complementar o CrossFit que ele já pratica, sem repetir a sobrecarga de coluna dos WODs. A corrida no sábado e o condicionamento são a atividade extra que acelera o gasto calórico e melhora o cardio. O que sustenta o resultado é constância, técnica impecável e progressão de carga semana a semana.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Correr 5 km contínuos sem parar=0; Ganhar massa em peito, costas e pernas=0</t>
+          <t>Reduzir o percentual de gordura=0; Ganhar massa muscular complementando o CrossFit=0</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -6606,7 +6606,6 @@
           <t>Corrida · aquecimento</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
           <t>5 min</t>
@@ -6644,7 +6643,6 @@
           <t>Corrida · Semana 1</t>
         </is>
       </c>
-      <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
           <t>4-5 km</t>
@@ -6724,7 +6722,6 @@
           <t>Corrida · Semana 3</t>
         </is>
       </c>
-      <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
           <t>5-6 km</t>
@@ -6762,7 +6759,6 @@
           <t>Corrida · Semana 4</t>
         </is>
       </c>
-      <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
           <t>5 km</t>
@@ -6800,7 +6796,6 @@
           <t>Corrida · volta à calma</t>
         </is>
       </c>
-      <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
           <t>5 min</t>

</xml_diff>

<commit_message>
Ajustes no treino do Nilo (dias A, B e C)
A: inclui crucifixo halteres no banco inclinado, elevacao lateral em 3 series,
   remove face pull, reordena peito>ombro>triceps
B: inclui remada alta no pulley (barra V/W), crucifixo inverso no banco com halteres
C: remove serratus punch, inclui abducao horizontal unilateral e pulldown barra reta

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -983,7 +983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J142"/>
+  <dimension ref="A1:J144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4313,12 +4313,12 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Peck deck</t>
+          <t>Crucifixo com halteres no banco inclinado</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Peitoral</t>
+          <t>Peitoral superior</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -4328,12 +4328,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Banco inclinado: abre os halteres sentindo o peito alongar, sobe controlado sem bater os halteres no topo.</t>
         </is>
       </c>
     </row>
@@ -4355,17 +4355,17 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Elevação lateral</t>
+          <t>Peck deck</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Deltóide lateral</t>
+          <t>Peitoral</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -4397,7 +4397,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Elevação lateral no cabo</t>
+          <t>Elevação lateral</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4412,12 +4412,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Segura 1 seg no topo (isometria).</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -4439,12 +4439,12 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Face pull</t>
+          <t>Elevação lateral no cabo</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Deltóide posterior</t>
+          <t>Deltóide lateral</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -4459,7 +4459,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Saúde do ombro: cotovelos altos, segura 1 seg na contração.</t>
+          <t>Segura 1 seg no topo (isometria).</t>
         </is>
       </c>
     </row>
@@ -4686,12 +4686,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Crucifixo inverso</t>
+          <t>Remada alta no pulley com barra V ou W</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Deltóide posterior</t>
+          <t>Trapézio / deltoide</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4701,7 +4701,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12-15</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Puxa a barra até a altura do peito, cotovelos altos e acima das mãos, sem encolher os ombros.</t>
         </is>
       </c>
     </row>
@@ -4723,27 +4728,27 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Rosca direta + rosca martelo (bi-set)</t>
+          <t>Crucifixo inverso no banco com halteres</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Bíceps</t>
+          <t>Deltóide posterior</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>12 cada</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Bi-set: as duas roscas em sequência, sem descanso entre elas.</t>
+          <t>Peito apoiado no banco inclinado, abre os halteres apertando as escápulas. Deltoide posterior, carga moderada.</t>
         </is>
       </c>
     </row>
@@ -4765,7 +4770,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Rosca scott (banco)</t>
+          <t>Rosca direta + rosca martelo (bi-set)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4775,17 +4780,17 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>12 cada</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Bi-set: as duas roscas em sequência, sem descanso entre elas.</t>
         </is>
       </c>
     </row>
@@ -4797,22 +4802,22 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>C · Qua · Manguito e Estabilização</t>
+          <t>B · Ter · Costas e Bíceps</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Rotação externa a 90° (cabo ou elástico)</t>
+          <t>Rosca scott (banco)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Manguito rotador</t>
+          <t>Bíceps</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4822,12 +4827,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>12 cada</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Braço a 90°: fortalece o manguito na posição de overhead do CrossFit.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -4849,7 +4854,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Rotação interna no cabo</t>
+          <t>Rotação externa a 90° (cabo ou elástico)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4864,12 +4869,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>15 cada</t>
+          <t>12 cada</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Equilíbrio do manguito (subescapular).</t>
+          <t>Braço a 90°: fortalece o manguito na posição de overhead do CrossFit.</t>
         </is>
       </c>
     </row>
@@ -4891,12 +4896,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Face pull</t>
+          <t>Rotação interna no cabo</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Estabilizadores da escápula</t>
+          <t>Manguito rotador</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4906,12 +4911,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15 cada</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>Retração escapular, cotovelos altos. Segura 1 seg na contração (isometria).</t>
+          <t>Equilíbrio do manguito (subescapular).</t>
         </is>
       </c>
     </row>
@@ -4933,12 +4938,12 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Band pull-apart (abertura com elástico)</t>
+          <t>Face pull</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Trapézio médio/posterior</t>
+          <t>Estabilizadores da escápula</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -4948,12 +4953,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>15-20</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>Abre o elástico à frente do corpo juntando as escápulas. Prehab de ombro, carga leve.</t>
+          <t>Retração escapular, cotovelos altos. Segura 1 seg na contração (isometria).</t>
         </is>
       </c>
     </row>
@@ -4975,12 +4980,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Serrátil (serratus punch no cabo)</t>
+          <t>Band pull-apart (abertura com elástico)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Serrátil anterior</t>
+          <t>Trapézio médio/posterior</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4990,12 +4995,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15-20</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Empurra e 'avança' a escápula no final do movimento.</t>
+          <t>Abre o elástico à frente do corpo juntando as escápulas. Prehab de ombro, carga leve.</t>
         </is>
       </c>
     </row>
@@ -5017,12 +5022,12 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Pallof press no cabo</t>
+          <t>Abdução horizontal de ombros unilateral na polia</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Core · anti-rotação</t>
+          <t>Deltóide posterior</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -5037,7 +5042,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Segura 2 seg na ponta (isometria anti-rotação). Tronco firme.</t>
+          <t>Um braço de cada vez, braço estendido levando a polia pra fora na horizontal. Deltoide posterior e estabilidade do ombro, carga leve e controlado.</t>
         </is>
       </c>
     </row>
@@ -5059,12 +5064,12 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Prancha com toque no ombro</t>
+          <t>Pulldown na polia com barra reta (braços estendidos)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Core · estabilização</t>
+          <t>Dorsal / serrátil</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -5074,12 +5079,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>20 toques</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Quadril estável, sem balançar. 20 toques no total.</t>
+          <t>Braços estendidos, puxa a barra até as coxas com o dorsal e o serrátil, sem dobrar o cotovelo. Controla a volta.</t>
         </is>
       </c>
     </row>
@@ -5091,37 +5096,37 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>D · Qui · Quadríceps</t>
+          <t>C · Qua · Manguito e Estabilização</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Hack squat</t>
+          <t>Pallof press no cabo</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Core · anti-rotação</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>15/12/10/08</t>
+          <t>12 cada</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>Progressão de carga. Único composto do dia (o agacho pesado já vem do CrossFit).</t>
+          <t>Segura 2 seg na ponta (isometria anti-rotação). Tronco firme.</t>
         </is>
       </c>
     </row>
@@ -5133,37 +5138,37 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>D · Qui · Quadríceps</t>
+          <t>C · Qua · Manguito e Estabilização</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Cadeira extensora</t>
+          <t>Prancha com toque no ombro</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Core · estabilização</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>20 toques</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso; segura 1 seg no topo de cada rep.</t>
+          <t>Quadril estável, sem balançar. 20 toques no total.</t>
         </is>
       </c>
     </row>
@@ -5185,27 +5190,27 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Mesa flexora</t>
+          <t>Hack squat</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15/12/10/08</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2 min de isometria ao final da última série.</t>
+          <t>Progressão de carga. Único composto do dia (o agacho pesado já vem do CrossFit).</t>
         </is>
       </c>
     </row>
@@ -5227,27 +5232,27 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Cadeira adutora</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Adutores</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>15 ISO + 15</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>15 seg de isometria + 15 reps por série.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso; segura 1 seg no topo de cada rep.</t>
         </is>
       </c>
     </row>
@@ -5269,27 +5274,27 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Panturrilha em pé</t>
+          <t>Mesa flexora</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Panturrilha</t>
+          <t>Posterior</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>20/15/12/12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Progressão de carga. Amplitude total.</t>
+          <t>2 min de isometria ao final da última série.</t>
         </is>
       </c>
     </row>
@@ -5311,12 +5316,12 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Panturrilha sentada</t>
+          <t>Cadeira adutora</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Panturrilha</t>
+          <t>Adutores</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -5326,7 +5331,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15 ISO + 15</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>15 seg de isometria + 15 reps por série.</t>
         </is>
       </c>
     </row>
@@ -5338,22 +5348,22 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>E · Sáb · Pontos Fracos</t>
+          <t>D · Qui · Quadríceps</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Elevação lateral</t>
+          <t>Panturrilha em pé</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Deltóide lateral</t>
+          <t>Panturrilha</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -5363,12 +5373,12 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>20/15/12</t>
+          <t>20/15/12/12</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (20 → 15 → 12) até a falha.</t>
+          <t>Progressão de carga. Amplitude total.</t>
         </is>
       </c>
     </row>
@@ -5380,22 +5390,22 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>E · Sáb · Pontos Fracos</t>
+          <t>D · Qui · Quadríceps</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Elevação lateral no cabo (unilateral)</t>
+          <t>Panturrilha sentada</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Deltóide lateral</t>
+          <t>Panturrilha</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -5405,12 +5415,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>Carga leve, um braço de cada vez, controla a descida.</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -5432,27 +5437,27 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Crucifixo inverso</t>
+          <t>Elevação lateral</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Deltóide posterior</t>
+          <t>Deltóide lateral</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>20/15/12</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Ombro posterior: aperta as escápulas no fim do movimento.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (20 → 15 → 12) até a falha.</t>
         </is>
       </c>
     </row>
@@ -5474,12 +5479,12 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Rosca direta + tríceps na corda (bi-set)</t>
+          <t>Elevação lateral no cabo (unilateral)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Bíceps/tríceps</t>
+          <t>Deltóide lateral</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -5489,12 +5494,12 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>15 cada</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Bi-set: um logo após o outro, sem descanso.</t>
+          <t>Carga leve, um braço de cada vez, controla a descida.</t>
         </is>
       </c>
     </row>
@@ -5516,12 +5521,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Rosca martelo</t>
+          <t>Crucifixo inverso</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Bíceps</t>
+          <t>Deltóide posterior</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -5531,12 +5536,12 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Pegada neutra, cotovelo fixo junto ao corpo.</t>
+          <t>Ombro posterior: aperta as escápulas no fim do movimento.</t>
         </is>
       </c>
     </row>
@@ -5558,12 +5563,12 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Tríceps testa</t>
+          <t>Rosca direta + tríceps na corda (bi-set)</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Tríceps</t>
+          <t>Bíceps/tríceps</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -5573,12 +5578,12 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15 cada</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Cotovelos apontados pra frente, controla a descida.</t>
+          <t>Bi-set: um logo após o outro, sem descanso.</t>
         </is>
       </c>
     </row>
@@ -5600,12 +5605,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Panturrilha em pé</t>
+          <t>Rosca martelo</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Panturrilha</t>
+          <t>Bíceps</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -5615,12 +5620,12 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Segura 2 seg no topo (isometria).</t>
+          <t>Pegada neutra, cotovelo fixo junto ao corpo.</t>
         </is>
       </c>
     </row>
@@ -5642,12 +5647,12 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Panturrilha sentada</t>
+          <t>Tríceps testa</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Panturrilha</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -5657,7 +5662,12 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Cotovelos apontados pra frente, controla a descida.</t>
         </is>
       </c>
     </row>
@@ -5679,12 +5689,12 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Abdominal na corda no pulley</t>
+          <t>Panturrilha em pé</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Panturrilha</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -5694,7 +5704,12 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Segura 2 seg no topo (isometria).</t>
         </is>
       </c>
     </row>
@@ -5716,12 +5731,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Prancha</t>
+          <t>Panturrilha sentada</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Panturrilha</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -5731,96 +5746,86 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>40s</t>
-        </is>
-      </c>
-      <c r="I116" t="inlineStr">
-        <is>
-          <t>Isometria: corpo alinhado, abdômen contraído.</t>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>A · Ter · Peito</t>
+          <t>E · Sáb · Pontos Fracos</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Supino na máquina (chest press)</t>
+          <t>Abdominal na corda no pulley</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Peitoral · principal</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>12/10/8/8</t>
-        </is>
-      </c>
-      <c r="I117" t="inlineStr">
-        <is>
-          <t>Progressão de carga ao longo das séries. Empurra controlado, sem travar o cotovelo no fim.</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Felipe</t>
+          <t>Nilo Sheeny</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>A · Ter · Peito</t>
+          <t>E · Sáb · Pontos Fracos</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Supino inclinado com halteres</t>
+          <t>Prancha</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Peitoral</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>40s</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Progressão de carga: aumente o peso a cada série mantendo a técnica.</t>
+          <t>Isometria: corpo alinhado, abdômen contraído.</t>
         </is>
       </c>
     </row>
@@ -5842,27 +5847,27 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Crucifixo na máquina (voador)</t>
+          <t>Supino na máquina (chest press)</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Peitoral</t>
+          <t>Peitoral · principal</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>12/10/8/8</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Abre bem e segura 1 seg na contração.</t>
+          <t>Progressão de carga ao longo das séries. Empurra controlado, sem travar o cotovelo no fim.</t>
         </is>
       </c>
     </row>
@@ -5884,7 +5889,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Crossover na polia</t>
+          <t>Supino inclinado com halteres</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -5894,17 +5899,17 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Progressão de carga: aumente o peso a cada série mantendo a técnica.</t>
         </is>
       </c>
     </row>
@@ -5926,12 +5931,12 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Tríceps na corda</t>
+          <t>Crucifixo na máquina (voador)</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Tríceps</t>
+          <t>Peitoral</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -5946,7 +5951,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Cotovelos fixos junto ao corpo, abre bem no fim.</t>
+          <t>Abre bem e segura 1 seg na contração.</t>
         </is>
       </c>
     </row>
@@ -5968,12 +5973,12 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Tríceps testa</t>
+          <t>Crossover na polia</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Tríceps</t>
+          <t>Peitoral</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -6000,37 +6005,37 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>B · Qui · Costas</t>
+          <t>A · Ter · Peito</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Barra fixa ou puxada alta (pegada aberta)</t>
+          <t>Tríceps na corda</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Costas · principal</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>12/10/8/8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Progressão de carga ao longo das séries.</t>
+          <t>Cotovelos fixos junto ao corpo, abre bem no fim.</t>
         </is>
       </c>
     </row>
@@ -6042,37 +6047,37 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>B · Qui · Costas</t>
+          <t>A · Ter · Peito</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Remada sentada na máquina (pegada neutra)</t>
+          <t>Tríceps testa</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Tríceps</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>12/10/10/08</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Progressão de carga. Controla a fase negativa.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -6094,27 +6099,27 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Remada cavalinho (T-bar)</t>
+          <t>Barra fixa ou puxada alta (pegada aberta)</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Costas · principal</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>10-12</t>
+          <t>12/10/8/8</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Peito apoiado, puxa com os cotovelos.</t>
+          <t>Progressão de carga ao longo das séries.</t>
         </is>
       </c>
     </row>
@@ -6136,7 +6141,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Puxada com triângulo (pegada neutra)</t>
+          <t>Remada sentada na máquina (pegada neutra)</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -6146,17 +6151,17 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>12/10/10/08</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Leva o triângulo ao peito, escápulas pra baixo.</t>
+          <t>Progressão de carga. Controla a fase negativa.</t>
         </is>
       </c>
     </row>
@@ -6178,7 +6183,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Pullover na polia</t>
+          <t>Remada cavalinho (T-bar)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -6193,12 +6198,12 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10-12</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Sente o dorsal alongar e contrair, cotovelos semi-fixos.</t>
+          <t>Peito apoiado, puxa com os cotovelos.</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6225,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Remada unilateral com halter (serrote)</t>
+          <t>Puxada com triângulo (pegada neutra)</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -6235,12 +6240,12 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>10 cada</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Um lado de cada vez, sem rodar o tronco.</t>
+          <t>Leva o triângulo ao peito, escápulas pra baixo.</t>
         </is>
       </c>
     </row>
@@ -6262,12 +6267,12 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Rosca scott (banco)</t>
+          <t>Pullover na polia</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Bíceps</t>
+          <t>Costas</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -6277,12 +6282,12 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>10-12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Progressão de carga: aumente o peso a cada série. Cotovelos apoiados no banco, sobe e desce controlado.</t>
+          <t>Sente o dorsal alongar e contrair, cotovelos semi-fixos.</t>
         </is>
       </c>
     </row>
@@ -6294,37 +6299,37 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>C · Sex · Pernas</t>
+          <t>B · Qui · Costas</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Leg press 45°</t>
+          <t>Remada unilateral com halter (serrote)</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Pernas · principal</t>
+          <t>Costas</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>12/10/10/08</t>
+          <t>10 cada</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Progressão de carga. Pés na largura do quadril, desce controlado.</t>
+          <t>Um lado de cada vez, sem rodar o tronco.</t>
         </is>
       </c>
     </row>
@@ -6336,22 +6341,22 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>C · Sex · Pernas</t>
+          <t>B · Qui · Costas</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Agachamento hack</t>
+          <t>Rosca scott (banco)</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Bíceps</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -6366,7 +6371,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Máquina, poupando a coluna que o CrossFit já castiga.</t>
+          <t>Progressão de carga: aumente o peso a cada série. Cotovelos apoiados no banco, sobe e desce controlado.</t>
         </is>
       </c>
     </row>
@@ -6388,27 +6393,27 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Cadeira extensora</t>
+          <t>Leg press 45°</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
+          <t>Pernas · principal</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>12/10/10/08</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
+          <t>Progressão de carga. Pés na largura do quadril, desce controlado.</t>
         </is>
       </c>
     </row>
@@ -6430,27 +6435,27 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Mesa flexora (posterior)</t>
+          <t>Agachamento hack</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>12/10/10/10</t>
+          <t>10-12</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Progressão de carga. Controla a fase negativa.</t>
+          <t>Máquina, poupando a coluna que o CrossFit já castiga.</t>
         </is>
       </c>
     </row>
@@ -6472,12 +6477,12 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Coice de glúteo na polia</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Glúteos</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -6487,12 +6492,12 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>12 cada</t>
+          <t>15/12/10</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Um lado de cada vez, segura 1 seg na contração do glúteo.</t>
+          <t>Drop set: tudo na MESMA série, reduz a carga sem descanso (15 → 12 → 10) até a falha.</t>
         </is>
       </c>
     </row>
@@ -6514,27 +6519,27 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Elevação pélvica (glúteo)</t>
+          <t>Mesa flexora (posterior)</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Glúteos</t>
+          <t>Posterior</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>12/10/10/10</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Segura 2 seg no topo (isometria) apertando o glúteo.</t>
+          <t>Progressão de carga. Controla a fase negativa.</t>
         </is>
       </c>
     </row>
@@ -6556,27 +6561,27 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Panturrilha em pé</t>
+          <t>Coice de glúteo na polia</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Panturrilha</t>
+          <t>Glúteos</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>20/15/12/12</t>
+          <t>12 cada</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Drop set na última série + isometria de 2 seg no topo de cada rep.</t>
+          <t>Um lado de cada vez, segura 1 seg na contração do glúteo.</t>
         </is>
       </c>
     </row>
@@ -6588,32 +6593,37 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>D · Sáb · Corrida</t>
+          <t>C · Sex · Pernas</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Aquecimento</t>
+          <t>Elevação pélvica (glúteo)</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Corrida · aquecimento</t>
+          <t>Glúteos</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Faça o aquecimento, depois SÓ o bloco da semana atual do seu ciclo, e termine no desaquecimento. A cada 4 semanas o ciclo recomeça, subindo cerca de 10%. Comece com caminhada rápida evoluindo para trote leve.</t>
+          <t>Segura 2 seg no topo (isometria) apertando o glúteo.</t>
         </is>
       </c>
     </row>
@@ -6625,32 +6635,37 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>D · Sáb · Corrida</t>
+          <t>C · Sex · Pernas</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Semana 1 · Corrida contínua leve</t>
+          <t>Panturrilha em pé</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Corrida · Semana 1</t>
+          <t>Panturrilha</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>4-5 km</t>
+          <t>20/15/12/12</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Ritmo de conversa (Z2): você consegue falar frases inteiras. Registre seu tempo total no fim.</t>
+          <t>Drop set na última série + isometria de 2 seg no topo de cada rep.</t>
         </is>
       </c>
     </row>
@@ -6672,27 +6687,22 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Semana 2 · Fartlek</t>
+          <t>Aquecimento</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Corrida · Semana 2</t>
-        </is>
-      </c>
-      <c r="F139" t="inlineStr">
-        <is>
-          <t>6</t>
+          <t>Corrida · aquecimento</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>(3 min corrida + 1 min caminhada)</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>6 blocos de 3 min correndo moderado + 1 min caminhando. Registre o tempo total.</t>
+          <t>Faça o aquecimento, depois SÓ o bloco da semana atual do seu ciclo, e termine no desaquecimento. A cada 4 semanas o ciclo recomeça, subindo cerca de 10%. Comece com caminhada rápida evoluindo para trote leve.</t>
         </is>
       </c>
     </row>
@@ -6714,22 +6724,22 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Semana 3 · Longão leve</t>
+          <t>Semana 1 · Corrida contínua leve</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Corrida · Semana 3</t>
+          <t>Corrida · Semana 1</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>5-6 km</t>
+          <t>4-5 km</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Contínuo em Z2, sem pressa, construindo resistência. Registre seu tempo.</t>
+          <t>Ritmo de conversa (Z2): você consegue falar frases inteiras. Registre seu tempo total no fim.</t>
         </is>
       </c>
     </row>
@@ -6751,22 +6761,27 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Semana 4 · Progressiva</t>
+          <t>Semana 2 · Fartlek</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Corrida · Semana 4</t>
+          <t>Corrida · Semana 2</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>6</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>5 km</t>
+          <t>(3 min corrida + 1 min caminhada)</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Comece leve e termine o último km mais forte (limiar leve). Registre seu tempo.</t>
+          <t>6 blocos de 3 min correndo moderado + 1 min caminhando. Registre o tempo total.</t>
         </is>
       </c>
     </row>
@@ -6788,20 +6803,94 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
+          <t>Semana 3 · Longão leve</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Corrida · Semana 3</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>5-6 km</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Contínuo em Z2, sem pressa, construindo resistência. Registre seu tempo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>D · Sáb · Corrida</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Semana 4 · Progressiva</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Corrida · Semana 4</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>5 km</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Comece leve e termine o último km mais forte (limiar leve). Registre seu tempo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>D · Sáb · Corrida</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
           <t>Desaquecimento</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr">
+      <c r="E144" t="inlineStr">
         <is>
           <t>Corrida · volta à calma</t>
         </is>
       </c>
-      <c r="G142" t="inlineStr">
+      <c r="G144" t="inlineStr">
         <is>
           <t>5 min</t>
         </is>
       </c>
-      <c r="I142" t="inlineStr">
+      <c r="I144" t="inlineStr">
         <is>
           <t>Trote bem leve até virar caminhada, depois alongue panturrilha, posterior e quadril.</t>
         </is>

</xml_diff>

<commit_message>
Adiciona Treino D (circuito full body) da Jaqueline, frequência 4x/semana
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -690,7 +690,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Foco: ganho de massa muscular e força em membros inferiores · Treinos A, B e C</t>
+          <t>Foco: ganho de massa muscular e força em membros inferiores · Treinos A, B, C e D</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Evolução excelente desde 05/2025: saiu de 32% para 18,8% de gordura, com ótima recomposição corporal. Novo ciclo com foco em ganho de massa muscular e força em membros inferiores, com técnica impecável e progressão de carga. Treinos A (quadríceps), B (superiores, com bi-sets) e C (posterior/glúteos).</t>
+          <t>Evolução excelente desde 05/2025: saiu de 32% para 18,8% de gordura, com ótima recomposição corporal. Novo ciclo com foco em ganho de massa muscular e força em membros inferiores, com técnica impecável e progressão de carga. Treinos A (quadríceps), B (superiores, com bi-sets), C (posterior/glúteos) e D (circuito full body).</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N3" t="n">
@@ -983,7 +983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J140"/>
+  <dimension ref="A1:J145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6720,6 +6720,196 @@
       <c r="G140" t="inlineStr">
         <is>
           <t>2 min leve / 2 min forte × 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>D · Circuito Full Body</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Flexão de braço de joelhos</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Peito/Core</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Circuito: repetir os 5 exercícios em sequência, 3 voltas — 30s de descanso entre exercícios e 2 min entre as voltas. Sem carga (peso do corpo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>D · Circuito Full Body</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Step-up no box</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Pernas/glúteos</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>10 cada perna</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>D · Circuito Full Body</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Senta e levanta com halteres no box</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Pernas/glúteos</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>D · Circuito Full Body</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Mountain climber no box</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Cardio</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>40s</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Jaqueline Galo</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>D · Circuito Full Body</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Abdominal curto no solo</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige rodagem da Lara pra 4km e recuperacao do tiro (parada na lateral da esteira)
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -6351,7 +6351,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Tiro de 800m em ritmo forte (bem acima do confortável, quase máximo sustentável). Recuperação de 2-3 min em trote leve/caminhada entre os tiros. Repita 4x.</t>
+          <t>Tiro de 800m em ritmo forte (bem acima do confortável, quase máximo sustentável). Recuperação de 2-3 min parado na lateral da esteira entre os tiros. Repita 4x.</t>
         </is>
       </c>
     </row>
@@ -6835,7 +6835,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>3 km</t>
+          <t>4 km</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">

</xml_diff>

<commit_message>
Lara: novo ciclo A-D (emagrecimento + condicionamento aeróbico, tiros na esteira)
</commit_message>
<xml_diff>
--- a/gerador/modelo-treinos.xlsx
+++ b/gerador/modelo-treinos.xlsx
@@ -750,17 +750,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Foco: condicionamento fisico e massa magra · Treinos A–F (seg a sáb)</t>
+          <t>Foco: emagrecimento e condicionamento aeróbico · Treinos A-D</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MELHORA DO CONDICIONAMENTO FÍSICO E AUMENTO DE MASSA MAGRA</t>
+          <t>EMAGRECIMENTO E CONDICIONAMENTO AERÓBICO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Atleta experiente em musculação, retomando a corrida de forma estruturada. Objetivo principal: melhora do condicionamento físico (capacidade aeróbica e resistência); meta secundária: aumento de massa magra. Ciclo de 6 dias combinando musculação (Inferiores/Superiores/Posterior) com 3 estímulos de corrida distintos: tiro (velocidade), rodagem (base aeróbica) e fartlek (variação de ritmo).</t>
+          <t>Atleta experiente em musculação, agora com foco em perda de gordura e melhora do condicionamento aeróbico. Treino em formato metabólico: séries de reps altas, circuitos com bi-sets e tiros de 800m na esteira, além de HIIT na bike e corrida contínua. Prioridade em densidade de treino e gasto calórico, mantendo estímulo de carga nos inferiores para preservar massa magra. Frequência de pelo menos 4x por semana.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -785,11 +785,11 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -983,7 +983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J150"/>
+  <dimension ref="A1:J138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5748,32 +5748,27 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>A · Inferiores</t>
+          <t>A · Tiros longos na esteira + core</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Agachamento no Hack</t>
+          <t>Esteira — aquecimento progressivo</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Pernas/glúteos · principal</t>
-        </is>
-      </c>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>4</t>
+          <t>Cardio · aquecimento</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>15/12/10/08</t>
+          <t>10 min</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Progressão de carga ao longo das séries (pirâmide).</t>
+          <t>Comece em caminhada e aumente o ritmo aos poucos até um trote confortável, preparando o corpo para os tiros.</t>
         </is>
       </c>
     </row>
@@ -5790,17 +5785,17 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>A · Inferiores</t>
+          <t>A · Tiros longos na esteira + core</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Leg press 45°</t>
+          <t>Esteira — tiros de 800m</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Pernas</t>
+          <t>Cardio · intervalado</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -5810,12 +5805,12 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>800m forte</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Não estender totalmente os joelhos no topo; descida controlada.</t>
+          <t>Cada tiro de 800m em ritmo forte, bem acima do confortável. Recuperação de 2–3 min em caminhada entre os tiros. Repita 4x.</t>
         </is>
       </c>
     </row>
@@ -5832,32 +5827,27 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>A · Inferiores</t>
+          <t>A · Tiros longos na esteira + core</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Cadeira extensora</t>
+          <t>Esteira — desaquecimento</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Quadríceps</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>3</t>
+          <t>Cardio · desaquecimento</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>15/12/10</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Progressão de carga ao longo das séries (pirâmide).</t>
+          <t>Trote leve reduzindo o ritmo aos poucos. Finalize com alongamento de pernas.</t>
         </is>
       </c>
     </row>
@@ -5874,17 +5864,17 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>A · Inferiores</t>
+          <t>A · Tiros longos na esteira + core</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Cadeira flexora</t>
+          <t>Prancha abdominal</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Posterior de coxa</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -5894,12 +5884,12 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1 min</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Movimento controlado, segurar 1s na contração.</t>
+          <t>Corpo alinhado da cabeça ao calcanhar, abdômen contraído.</t>
         </is>
       </c>
     </row>
@@ -5916,17 +5906,17 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>A · Inferiores</t>
+          <t>A · Tiros longos na esteira + core</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Panturrilha em pé livre</t>
+          <t>Abdominal oblíquo (bicicleta)</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Panturrilha · tríceps sural</t>
+          <t>Core · oblíquos</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -5937,6 +5927,11 @@
       <c r="G121" t="inlineStr">
         <is>
           <t>20</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Alterne cotovelo–joelho oposto, movimento controlado, sem puxar o pescoço.</t>
         </is>
       </c>
     </row>
@@ -5948,22 +5943,22 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>A · Inferiores</t>
+          <t>B · Inferiores</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Bike — HIIT</t>
+          <t>Leg press horizontal</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Cardio · intervalado</t>
+          <t>Pernas · principal</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -5973,12 +5968,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2 min forte + 3 min lento</t>
+          <t>15/12/10/08</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>HIIT na bike: 4 blocos de 2 min em ritmo forte (alta intensidade) + 3 min em ritmo lento (recuperação ativa). Repita os 4 blocos (~20 min no total).</t>
+          <t>Progressão de carga ao longo das séries (pirâmide): aumenta a carga e diminui as reps a cada série.</t>
         </is>
       </c>
     </row>
@@ -5995,17 +5990,17 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>B · Superiores e Core</t>
+          <t>B · Inferiores</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Puxador frente com triângulo</t>
+          <t>Cadeira extensora</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Dorsais · principal</t>
+          <t>Quadríceps</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -6015,12 +6010,12 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Pegada triângulo (delta). Puxar com os cotovelos, levando até o peito.</t>
+          <t>Movimento controlado, sem dar impulso; segure meio segundo no topo.</t>
         </is>
       </c>
     </row>
@@ -6037,17 +6032,17 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>B · Superiores e Core</t>
+          <t>B · Inferiores</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Remada sentada na polia (pulley)</t>
+          <t>Cadeira flexora</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Costas</t>
+          <t>Posterior de coxa</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -6057,12 +6052,12 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Puxar próximo ao abdômen, peito aberto e coluna neutra.</t>
+          <t>Movimento controlado, segurar 1s na contração.</t>
         </is>
       </c>
     </row>
@@ -6079,17 +6074,17 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>B · Superiores e Core</t>
+          <t>B · Inferiores</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Supino sentado na máquina</t>
+          <t>Panturrilha em pé na máquina</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Peitoral</t>
+          <t>Panturrilha · tríceps sural</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -6099,12 +6094,12 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Controlar a descida, sem travar os cotovelos no final.</t>
+          <t>Amplitude total, subir bem no topo e segurar 1s.</t>
         </is>
       </c>
     </row>
@@ -6121,32 +6116,32 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>B · Superiores e Core</t>
+          <t>B · Inferiores</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Desenvolvimento com halteres</t>
+          <t>Bike — HIIT</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Ombro · principal</t>
+          <t>Cardio · intervalado</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>3 min pesado + 2 min devagar</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Core firme, sem arquear a lombar. Não travar os cotovelos no topo.</t>
+          <t>6 tiros: 3 min em ritmo pesado + 2 min devagar sem carga (recuperação ativa). Repita os 6 blocos (~30 min no total).</t>
         </is>
       </c>
     </row>
@@ -6158,22 +6153,22 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>B · Superiores e Core</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Prancha abdominal</t>
+          <t>Puxador frente delta + Rosca direta (bi-set)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Dorsais · bíceps</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -6183,12 +6178,12 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>1 min</t>
+          <t>15 / 20</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Corpo alinhado da cabeça ao calcanhar, abdômen contraído.</t>
+          <t>Bi-set sem descanso: puxador frente com pegada delta 15 reps, emenda rosca direta com halteres 20 reps. Descanse e repita 4x.</t>
         </is>
       </c>
     </row>
@@ -6200,37 +6195,37 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>B · Superiores e Core</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Abdominal curto no solo</t>
+          <t>Esteira — 800m</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Cardio · intervalado</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>800m forte</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Contraia o abdômen no topo, sem puxar o pescoço.</t>
+          <t>Tiro de 800m em ritmo forte logo depois do bi-set.</t>
         </is>
       </c>
     </row>
@@ -6242,22 +6237,22 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>B · Superiores e Core</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Bike — HIIT</t>
+          <t>Remada sentada + Desenvolvimento com halteres em pé (bi-set)</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Cardio · intervalado</t>
+          <t>Costas · ombro</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -6267,12 +6262,12 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2 min forte + 3 min lento</t>
+          <t>15 cada</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>HIIT na bike: 4 blocos de 2 min em ritmo forte (alta intensidade) + 3 min em ritmo lento (recuperação ativa). Repita os 4 blocos (~20 min no total).</t>
+          <t>Bi-set sem descanso: remada sentada 15 reps, emenda desenvolvimento com halteres em pé 15 reps. Repita 4x.</t>
         </is>
       </c>
     </row>
@@ -6289,27 +6284,32 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>C · Tiro + Braços/Ombros</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Corrida — aquecimento (trote leve)</t>
+          <t>Esteira — 800m</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Cardio · aquecimento</t>
+          <t>Cardio · intervalado</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>800m forte</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Trote leve, respiração tranquila, preparar o corpo para os tiros.</t>
+          <t>Tiro de 800m em ritmo forte.</t>
         </is>
       </c>
     </row>
@@ -6326,17 +6326,17 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>C · Tiro + Braços/Ombros</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Pista — tiros de 800m</t>
+          <t>Supino sentado na máquina + Tríceps francês com halteres (bi-set)</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Cardio · intervalado</t>
+          <t>Peitoral · tríceps</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -6346,12 +6346,12 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>800m forte</t>
+          <t>15 cada</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Tiro de 800m em ritmo forte (bem acima do confortável, quase máximo sustentável). Recuperação de 2-3 min parado na lateral da esteira entre os tiros. Repita 4x.</t>
+          <t>Bi-set sem descanso: supino sentado na máquina 15 reps, emenda tríceps francês com halteres 15 reps. Repita 4x.</t>
         </is>
       </c>
     </row>
@@ -6368,27 +6368,32 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>C · Tiro + Braços/Ombros</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Corrida — desaquecimento (trote leve)</t>
+          <t>Esteira — 800m</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Cardio · desaquecimento</t>
+          <t>Cardio · intervalado</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>800m forte</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Trote leve diminuindo o ritmo aos poucos. Finalize com alongamento de pernas.</t>
+          <t>Último tiro de 800m em ritmo forte.</t>
         </is>
       </c>
     </row>
@@ -6405,32 +6410,32 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>C · Tiro + Braços/Ombros</t>
+          <t>C · Circuito de braço + tiros</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Rosca direta com halteres</t>
+          <t>Abdominal curto com peso</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Bíceps</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Cotovelos fixos junto ao corpo, sem balançar o tronco.</t>
+          <t>Segure o peso no peito, contraia o abdômen no topo sem puxar o pescoço.</t>
         </is>
       </c>
     </row>
@@ -6442,37 +6447,32 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>C · Tiro + Braços/Ombros</t>
+          <t>D · Corrida + glúteos</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Tríceps na polia com corda</t>
+          <t>Esteira — corrida contínua</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Tríceps</t>
-        </is>
-      </c>
-      <c r="F134" t="inlineStr">
-        <is>
-          <t>3</t>
+          <t>Cardio · aeróbico</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3 km sem parar</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Cotovelos fixos; abrir a corda no final do movimento.</t>
+          <t>Ritmo moderado e constante, sem pausa. Respiração controlada — dá pra manter conversa curta.</t>
         </is>
       </c>
     </row>
@@ -6484,37 +6484,37 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>C · Tiro + Braços/Ombros</t>
+          <t>D · Corrida + glúteos</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Desenvolvimento com halteres</t>
+          <t>Agachamento sumô com kettlebell</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Ombro · principal</t>
+          <t>Glúteos/pernas · principal</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Core firme, sem arquear a lombar. Não travar os cotovelos no topo.</t>
+          <t>Pés afastados e pontas abertas; desça mantendo o tronco ereto e o peso no calcanhar.</t>
         </is>
       </c>
     </row>
@@ -6526,27 +6526,27 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>C · Tiro + Braços/Ombros</t>
+          <t>D · Corrida + glúteos</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Elevação lateral</t>
+          <t>Cadeira abdutora</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Deltoide medial</t>
+          <t>Glúteos · abdutores</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Subir até a linha dos ombros, cotovelos levemente flexionados.</t>
+          <t>Abrir as pernas com controle, sem jogar o tronco para trás.</t>
         </is>
       </c>
     </row>
@@ -6573,17 +6573,17 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>D · Posterior, Glúteos e Lombar</t>
+          <t>D · Corrida + glúteos</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Stiff com halteres</t>
+          <t>Glúteo coice na polia</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Posterior de coxa · principal</t>
+          <t>Glúteos</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -6593,12 +6593,12 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Joelhos levemente flexionados; descer controlando até sentir o alongamento no posterior, mantendo a coluna neutra.</t>
+          <t>Movimento controlado; contraia o glúteo no topo sem hiperestender a lombar.</t>
         </is>
       </c>
     </row>
@@ -6615,17 +6615,17 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>D · Posterior, Glúteos e Lombar</t>
+          <t>D · Corrida + glúteos</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Cadeira flexora</t>
+          <t>Prancha abdominal</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Posterior de coxa</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -6635,486 +6635,12 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1 min</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Movimento controlado, segurar 1s na contração.</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>Lara</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>D · Posterior, Glúteos e Lombar</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>Cadeira abdutora</t>
-        </is>
-      </c>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t>Glúteos · abdutores</t>
-        </is>
-      </c>
-      <c r="F139" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G139" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="I139" t="inlineStr">
-        <is>
-          <t>Abrir as pernas com controle, sem jogar o tronco para trás.</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>Lara</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>D · Posterior, Glúteos e Lombar</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>Glúteo no cabo (coice)</t>
-        </is>
-      </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>Glúteos</t>
-        </is>
-      </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="I140" t="inlineStr">
-        <is>
-          <t>Movimento controlado; contraia o glúteo no topo sem hiperestender a lombar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>Lara</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>D · Posterior, Glúteos e Lombar</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t>Cadeira romana (extensão lombar)</t>
-        </is>
-      </c>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>Lombar · core</t>
-        </is>
-      </c>
-      <c r="F141" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G141" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="I141" t="inlineStr">
-        <is>
-          <t>Subir até alinhar o tronco; não hiperestender a lombar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>Lara</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>E · Rodagem</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>Corrida — aquecimento (caminhada)</t>
-        </is>
-      </c>
-      <c r="E142" t="inlineStr">
-        <is>
-          <t>Cardio · aquecimento</t>
-        </is>
-      </c>
-      <c r="G142" t="inlineStr">
-        <is>
-          <t>5 min</t>
-        </is>
-      </c>
-      <c r="I142" t="inlineStr">
-        <is>
-          <t>Caminhada leve (~5-6 km/h) para preparar o corpo. Respiração tranquila.</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>Lara</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>E · Rodagem</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>Corrida — rodagem contínua</t>
-        </is>
-      </c>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t>Cardio · aeróbico</t>
-        </is>
-      </c>
-      <c r="G143" t="inlineStr">
-        <is>
-          <t>4 km</t>
-        </is>
-      </c>
-      <c r="I143" t="inlineStr">
-        <is>
-          <t>Ritmo moderado e constante, sem parar. Respiração controlada — dá pra manter conversa curta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>Lara</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>E · Rodagem</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>Corrida — desaquecimento (caminhada)</t>
-        </is>
-      </c>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>Cardio · desaquecimento</t>
-        </is>
-      </c>
-      <c r="G144" t="inlineStr">
-        <is>
-          <t>5 min</t>
-        </is>
-      </c>
-      <c r="I144" t="inlineStr">
-        <is>
-          <t>Caminhada leve diminuindo o ritmo aos poucos. Finalize com alongamento de pernas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>Lara</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>F · Fartlek</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>Corrida — aquecimento (trote leve)</t>
-        </is>
-      </c>
-      <c r="E145" t="inlineStr">
-        <is>
-          <t>Cardio · aquecimento</t>
-        </is>
-      </c>
-      <c r="G145" t="inlineStr">
-        <is>
-          <t>5 min</t>
-        </is>
-      </c>
-      <c r="I145" t="inlineStr">
-        <is>
-          <t>Trote leve, preparar o corpo para o fartlek.</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>Lara</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>F · Fartlek</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>Corrida — fartlek</t>
-        </is>
-      </c>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>Cardio · intervalado</t>
-        </is>
-      </c>
-      <c r="G146" t="inlineStr">
-        <is>
-          <t>20 min</t>
-        </is>
-      </c>
-      <c r="I146" t="inlineStr">
-        <is>
-          <t>Corrida contínua com variações livres de ritmo: alterne blocos de ~1-2 min em ritmo forte com ~1-2 min de trote leve, conforme a sensação. Sem tempo fixo — o objetivo é variar a intensidade ao longo dos 20 min.</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>Lara</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>F · Fartlek</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>Corrida — desaquecimento (trote leve)</t>
-        </is>
-      </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>Cardio · desaquecimento</t>
-        </is>
-      </c>
-      <c r="G147" t="inlineStr">
-        <is>
-          <t>5 min</t>
-        </is>
-      </c>
-      <c r="I147" t="inlineStr">
-        <is>
-          <t>Trote leve diminuindo o ritmo aos poucos. Finalize com alongamento de pernas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>Lara</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>F · Fartlek</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>Abdominal infra (elevação de pernas)</t>
-        </is>
-      </c>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t>Core · infra</t>
-        </is>
-      </c>
-      <c r="F148" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="I148" t="inlineStr">
-        <is>
-          <t>Pernas estendidas, eleve controlando o balanço; não deixe a lombar arquear.</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>Lara</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>F · Fartlek</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>Abdominal oblíquo (bicicleta)</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>Core · oblíquos</t>
-        </is>
-      </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G149" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="I149" t="inlineStr">
-        <is>
-          <t>Alterne cotovelo-joelho oposto, movimento controlado, sem puxar o pescoço.</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>Lara</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>F · Fartlek</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>Prancha lateral</t>
-        </is>
-      </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>Core · lateral</t>
-        </is>
-      </c>
-      <c r="F150" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G150" t="inlineStr">
-        <is>
-          <t>30s cada lado</t>
-        </is>
-      </c>
-      <c r="I150" t="inlineStr">
-        <is>
-          <t>Corpo alinhado, quadril elevado e estável.</t>
+          <t>Corpo alinhado da cabeça ao calcanhar, abdômen contraído.</t>
         </is>
       </c>
     </row>
@@ -8296,17 +7822,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bloco 1 · Retomada</t>
+          <t>Bloco 1 · Adaptação metabólica</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CONSTÂNCIA E BASE</t>
+          <t>BASE AERÓBICA E CONSTÂNCIA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Reconstruir a constância e a técnica. Corrida no método caminhada-corrida.</t>
+          <t>Firmar a rotina de pelo menos 4 treinos por semana e a base de corrida. Tiros de 800m em ritmo controlado e circuitos com carga moderada, priorizando técnica e constância.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -8333,17 +7859,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bloco 2 · Hipertrofia metabólica</t>
+          <t>Bloco 2 · Densidade metabólica</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MASSA + GASTO</t>
+          <t>GASTO CALÓRICO</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Volume para preservar massa magra e densidade para o gasto calórico. Corrida progride.</t>
+          <t>Encurtar os descansos e subir o volume dos circuitos e do HIIT. Tiros de 800m mais fortes. Foco no gasto calórico mantendo a carga nos inferiores para preservar massa magra.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -8380,7 +7906,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Semana leve para recuperar.</t>
+          <t>Semana leve para recuperar antes do bloco mais intenso.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -8407,17 +7933,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bloco 3 · Definição</t>
+          <t>Bloco 3 · Pico de condicionamento</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>DENSIDADE</t>
+          <t>INTENSIDADE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Manter o músculo no déficit, corrida mais intensa.</t>
+          <t>Corrida mais intensa e circuitos no limite da densidade, segurando o músculo no déficit calórico.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -8454,7 +7980,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Reavaliação do percentual de gordura e ajustes do próximo ciclo.</t>
+          <t>Reavaliação do percentual de gordura e do condicionamento aeróbico; ajuste do próximo ciclo.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">

</xml_diff>